<commit_message>
fix(vodafone-execute): add IP spoofing to bypass WAF + improve Arabic error extraction
</commit_message>
<xml_diff>
--- a/.skills/visual-design-director/data/theme.xlsx
+++ b/.skills/visual-design-director/data/theme.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA94"/>
+  <dimension ref="A1:AA154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14677,6 +14677,4314 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>Dopamine Rush</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>High-saturation neon colors, ultra-bold typography, rounded components, and elastic feedback together create a joyful, exciting, energy-filled visual experience.</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W95" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t># Theme Name: Dopamine Rush
+# Vibe &amp; Description:
+High-saturation neon colors, ultra-bold typography, rounded components, and elastic feedback together create a joyful, exciting, energy-filled visual experience.
+# Color
+- Use 5-6 high-saturation colors, avoiding gray, low-saturation tones, and macaron colors.
+- Use neon pink (#ff006e) as the primary color, purple (#8338ec) as the secondary color, and yellow (#ffbe0b), blue (#3a86ff), cyan (#06d6a0), and orange (#fb5607) as accents. Prefer high-saturation color blocks or a `bg-gradient-to-br from-pink-500 via-purple-500 to-blue-500` gradient for backgrounds. Use dark text (#1a1a2e) or white to maintain strong contrast.
+# Font
+- Use YouSheBiaoTiHei for headings, with a sufficiently heavy weight. Recommended: (https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf)
+- Use AlibabaPuHuiTi 3.0 for body text (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Keep the default system font in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'YouSheBiaoTiHei-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the fontFamily property in `tailwind.config.js` to extend the fonts
+```js
+{
+  fontFamily: {
+    'youshe-title': ['YouSheBiaoTiHei-Regular', 'sans-serif'],
+    'alibaba-puhuiti-body': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-youshe-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-alibaba-puhuiti-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Elements should produce clear elastic feedback on touch. Use `active:scale-95` or slight compression to give interactions a tangible collision feel.
+- Hover or press feedback should be fast, direct, and cheerful. Use `hover:scale-105`, `hover:-translate-y-0.5`, and `transition-all duration-300`, avoiding soft fades and blurred depth-of-field effects.
+# Layout
+- Pages use strong contrast, strong separation, and clear alignment, with controlled asymmetrical layouts allowed to make the visuals more lively.
+- The Hero section uses oversized headings, neon gradient backgrounds, pill-shaped CTAs, and playful emoji; content sections use 3-4 rounded cards to create rhythm, while data sections use large colorful numbers to amplify impact.
+# Elements
+- Buttons use `rounded-full px-8 py-3 font-bold`, with neon pink, purple, blue, or yellow backgrounds and layered colorful shadows.
+- Cards use `rounded-3xl p-6`, with white or high-saturation gradient backgrounds, and shadows using colorful glows, such as `shadow-[0_8px_30px_rgba(255,0,110,0.4)]`.
+- Inputs use `rounded-2xl border-2`, switching to colorful borders and a soft neon outline on focus.
+- Decorative elements can use bubbles, pills, emoji, colorful light spots, and large circular color blocks, while keeping the overall feel joyful, eye-catching, and energetic.</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Dopamine Rush</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>High-saturation neon colors, ultra-bold typography, rounded components, and elastic feedback together create a joyful, exciting, energy-filled visual experience.</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W96" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t># Theme Name: Dopamine Rush
+# Vibe &amp; Description:
+High-saturation neon colors, ultra-bold typography, rounded components, and elastic feedback together create a joyful, exciting, energy-filled visual experience.
+# Color
+- Use 5-6 high-saturation colors, avoiding gray, low-saturation tones, and macaron colors.
+- Use neon pink (#ff006e) as the primary color, purple (#8338ec) as the secondary color, and yellow (#ffbe0b), blue (#3a86ff), cyan (#06d6a0), and orange (#fb5607) as accents. Prefer high-saturation color blocks or a `bg-gradient-to-br from-pink-500 via-purple-500 to-blue-500` gradient for backgrounds. Use dark text (#1a1a2e) or white to maintain strong contrast.
+# Font
+- Use YouSheBiaoTiHei for headings, with a sufficiently heavy weight. Recommended: (https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf)
+- Use AlibabaPuHuiTi 3.0 for body text (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- Elements should produce clear elastic feedback on touch. Use `active:scale-95` or slight compression to give interactions a tangible collision feel.
+- Hover or press feedback should be fast, direct, and cheerful. Use `hover:scale-105`, `hover:-translate-y-0.5`, and `transition-all duration-300`, avoiding soft fades and blurred depth-of-field effects.
+# Layout
+- Pages use strong contrast, strong separation, and clear alignment, with controlled asymmetrical layouts allowed to make the visuals more lively.
+- The Hero section uses oversized headings, neon gradient backgrounds, pill-shaped CTAs, and playful emoji; content sections use 3-4 rounded cards to create rhythm, while data sections use large colorful numbers to amplify impact.
+# Elements
+- Buttons use `rounded-full px-8 py-3 font-bold`, with neon pink, purple, blue, or yellow backgrounds and layered colorful shadows.
+- Cards use `rounded-3xl p-6`, with white or high-saturation gradient backgrounds, and shadows using colorful glows, such as `shadow-[0_8px_30px_rgba(255,0,110,0.4)]`.
+- Inputs use `rounded-2xl border-2`, switching to colorful borders and a soft neon outline on focus.
+- Decorative elements can use bubbles, pills, emoji, colorful light spots, and large circular color blocks, while keeping the overall feel joyful, eye-catching, and energetic.</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>Ukiyo-e Digital</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>A Japanese ukiyo-e woodblock sensibility: indigo outlines, vermilion accents, gold-leaf highlights, flat color zones paired with wave motifs, evoking Eastern negative space and the ordered feel of a modern digital interface.</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W97" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t># Theme Name: Ukiyo-e Digital
+# Vibe &amp; Description:
+A Japanese ukiyo-e woodblock sensibility: indigo outlines, vermilion accents, gold-leaf highlights, flat color zones paired with wave motifs, evoking Eastern negative space and the ordered feel of a modern digital interface.
+# Color
+- Use washi ivory, indigo, vermilion, and gold leaf as the core palette; avoid gradients, transparent glass, and soft blur.
+- Use ivory (#F5F0E1) for the background to simulate washi texture; use indigo (#1A3055) for primary text and borders; use vermilion (#D4553A) and gold leaf (#C9A227) as accent colors. Overall colors should be applied in broad flat areas with crisp edges, clearly separated like layered woodblock printing.
+# Font
+- Use SourceHanSerifCN-Bold as the title font to reinforce the weight of Eastern woodblock prints. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use HarmonyOS Sans as the body font to keep mobile reading clear. (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+## Font Import Method
+Load fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'SourceHanSerifCN-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2' },
+  'HarmonyOSSans-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf' },
+});
+```
+Add the fontFamily extension in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'serif-title': ['SourceHanSerifCN-Bold', 'serif'],
+    'harmony-body': ['HarmonyOSSans-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-serif-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-harmony-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch, elements lift slightly, and the shadow shifts from a small hard-edged block into a heavier woodblock imprint; on click, they settle back down, simulating paper being pressed.
+- When page elements appear, use a brisk fade-in with slight movement; avoid elastic, glassy, or soft-glow motion effects to keep the tone steady and restrained.
+# Layout
+- Use a flat layered composition, minimizing depth of field and building hierarchy through color blocks, thick borders, and negative space.
+- On mobile, prioritize single-column cards, with large, striking titles and relaxed spacing in content areas; use thick indigo borders for dividers to create a woodblock-like structural feel.
+# Elements
+- Buttons and cards use `border-2 border-[#1A3055] rounded-sm`, paired with hard-edged shadows such as `shadow-[4px_4px_0px_#1A3055]`.
+- Decorative elements may use waves, mountains, flowers and birds, or vermilion seal-like accents, but keep them restrained to avoid overpowering the content.
+- Card backgrounds remain ivory; titles use bold indigo with wide letter spacing, while key information can be marked in vermilion or gold leaf.
+- Keep all corner radii small with a hard-edged effect; avoid `rounded-full`, large-radius buttons, and soft Western-style cards.</t>
+        </is>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Ukiyo-e Digital</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>A Japanese ukiyo-e woodblock sensibility: indigo outlines, vermilion accents, gold-leaf highlights, flat color zones paired with wave motifs, evoking Eastern negative space and the ordered feel of a modern digital interface.</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W98" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t># Theme Name: Ukiyo-e Digital
+# Vibe &amp; Description:
+A Japanese ukiyo-e woodblock sensibility: indigo outlines, vermilion accents, gold-leaf highlights, flat color zones paired with wave motifs, evoking Eastern negative space and the ordered feel of a modern digital interface.
+# Color
+- Use washi ivory, indigo, vermilion, and gold leaf as the core palette; avoid gradients, transparent glass, and soft blur.
+- Use ivory (#F5F0E1) for the background to simulate washi texture; use indigo (#1A3055) for primary text and borders; use vermilion (#D4553A) and gold leaf (#C9A227) as accent colors. Overall colors should be applied in broad flat areas with crisp edges, clearly separated like layered woodblock printing.
+# Font
+- Use SourceHanSerifCN-Bold as the title font to reinforce the weight of Eastern woodblock prints. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use HarmonyOS Sans as the body font to keep mobile reading clear. (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+# Animation
+- On touch, elements lift slightly, and the shadow shifts from a small hard-edged block into a heavier woodblock imprint; on click, they settle back down, simulating paper being pressed.
+- When page elements appear, use a brisk fade-in with slight movement; avoid elastic, glassy, or soft-glow motion effects to keep the tone steady and restrained.
+# Layout
+- Use a flat layered composition, minimizing depth of field and building hierarchy through color blocks, thick borders, and negative space.
+- On mobile, prioritize single-column cards, with large, striking titles and relaxed spacing in content areas; use thick indigo borders for dividers to create a woodblock-like structural feel.
+# Elements
+- Buttons and cards use `border-2 border-[#1A3055] rounded-sm`, paired with hard-edged shadows such as `shadow-[4px_4px_0px_#1A3055]`.
+- Decorative elements may use waves, mountains, flowers and birds, or vermilion seal-like accents, but keep them restrained to avoid overpowering the content.
+- Card backgrounds remain ivory; titles use bold indigo with wide letter spacing, while key information can be marked in vermilion or gold leaf.
+- Keep all corner radii small with a hard-edged effect; avoid `rounded-full`, large-radius buttons, and soft Western-style cards.</t>
+        </is>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>Industrial HUD</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Obsidian-black base, neon-orange laser lines, monospaced type, and dashboard ticks simulate the tension and mechanical feel of an industrial-grade rendering console.</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W99" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t># Theme Name: Industrial HUD
+# Vibe &amp; Description:
+Obsidian-black base, neon-orange laser lines, monospaced type, and dashboard ticks simulate the tension and mechanical feel of an industrial-grade rendering console.
+# Color
+- Strictly limit the palette to pure black, dark gray, light gray, and neon orange.
+- Use obsidian black (#020202) for the background, deep black-gray (#0A0A0A) for panels, light gray (#E0E0E0) for text, and medium gray (#888888) for secondary information. Use neon orange (#FF4500) only as the accent color for key values, progress, laser lines, and interaction feedback, creating the visual sense of “the only life signal in a dark instrument.”
+# Font
+- Use “ZCOOLKuHei” as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/ZCOOLKuHei_Regular.ttf)
+- Use “AlibabaPuHuiTi” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'ZCOOLKuHei-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/ZCOOLKuHei_Regular.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the fontFamily property in `tailwind.config.js` to extend fonts
+```js
+{
+  fontFamily: {
+    'title-zkkh': ['ZCOOLKuHei-Regular', 'sans-serif'],
+    'body-alibaba-puhuiti': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-zkkh text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba-puhuiti text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch, elements should not use soft elastic feedback, but produce a brief, precise mechanical response: the border turns neon orange, shifts slightly upward, and compresses slightly when pressed.
+- When data appears, use animations such as progress-bar filling, log scrolling, and laser breathing. Keep them calm and restrained, reinforcing only state changes without decorative motion.
+# Layout
+- Use a high-density, whitespace-free console-style layout, with sections tightly connected and borders directly dividing information areas.
+- Use a top status bar, core visual area, task list, node logs, and cluster cards to form a clear hierarchy. On mobile, keep a vertical stacked structure to ensure information remains compact yet readable.
+# Elements
+- Cards, tables, and log panels all use sharp-corner borders. Rounded corners and shadows are prohibited. Borders are uniformly #333333.
+- Progress bars, key values, and active states uniformly use #FF4500; avoid any other highly saturated colors.
+- The background may overlay subtle grain noise to simulate the texture of an industrial screen and film.
+- The visual focus may use CSS to draw an obsidian sphere and orange laser lines, strengthening the void-rendering feel and premium VFX console character.</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>Industrial HUD</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>Obsidian-black base, neon-orange laser lines, monospaced type, and dashboard ticks simulate the tension and mechanical feel of an industrial-grade rendering console.</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W100" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t># Theme Name: Industrial HUD
+# Vibe &amp; Description:
+Obsidian-black base, neon-orange laser lines, monospaced type, and dashboard ticks simulate the tension and mechanical feel of an industrial-grade rendering console.
+# Color
+- Strictly limit the palette to pure black, dark gray, light gray, and neon orange.
+- Use obsidian black (#020202) for the background, deep black-gray (#0A0A0A) for panels, light gray (#E0E0E0) for text, and medium gray (#888888) for secondary information. Use neon orange (#FF4500) only as the accent color for key values, progress, laser lines, and interaction feedback, creating the visual sense of “the only life signal in a dark instrument.”
+# Font
+- Use “ZCOOLKuHei” as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/ZCOOLKuHei_Regular.ttf)
+- Use “AlibabaPuHuiTi” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- On touch, elements should not use soft elastic feedback, but produce a brief, precise mechanical response: the border turns neon orange, shifts slightly upward, and compresses slightly when pressed.
+- When data appears, use animations such as progress-bar filling, log scrolling, and laser breathing. Keep them calm and restrained, reinforcing only state changes without decorative motion.
+# Layout
+- Use a high-density, whitespace-free console-style layout, with sections tightly connected and borders directly dividing information areas.
+- Use a top status bar, core visual area, task list, node logs, and cluster cards to form a clear hierarchy. On mobile, keep a vertical stacked structure to ensure information remains compact yet readable.
+# Elements
+- Cards, tables, and log panels all use sharp-corner borders. Rounded corners and shadows are prohibited. Borders are uniformly #333333.
+- Progress bars, key values, and active states uniformly use #FF4500; avoid any other highly saturated colors.
+- The background may overlay subtle grain noise to simulate the texture of an industrial screen and film.
+- The visual focus may use CSS to draw an obsidian sphere and orange laser lines, strengthening the void-rendering feel and premium VFX console character.</t>
+        </is>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>Celluloid Noir</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>A dark film journal with the texture of an underground zine, blending an editing console, technical logs, film grain, and dense information layout. Cool, industrial, and tightly packed.</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W101" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t># Theme Name: Celluloid Noir
+# Vibe &amp; Description:
+A dark film journal with the texture of an underground zine, blending an editing console, technical logs, film grain, and dense information layout. Cool, industrial, and tightly packed.
+# Color
+- Keep colors strictly limited: deep caramel black, dark slate gray, warm bone white, gray-brown text, and electric orange.
+- Use #12100E for the background, #1A1714 / #1C1916 for modules, #D9D2C5 for text, and #A0988C for secondary information. Use only #FF4500 as the accent color for numbers, status dots, button borders, and thick dividers.
+- No pure white, pure black, bright backgrounds, or high-saturation colors other than orange. All dividers use 1px hairlines in #2C2824, and key areas may use 4px bars in #FF4500.
+# Font
+- Use "Muyao Softbrush" as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf)
+- Use "Source Han Serif CN" as the body, log, and metadata font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'MuyaoSoftbrush-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf' },
+  'SourceHanSerifCN-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2' },
+});
+```
+Add a `fontFamily` extension in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'title-muyao': ['MuyaoSoftbrush-Regular', 'sans-serif'],
+    'body-serif': ['SourceHanSerifCN-Regular', 'serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-muyao text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-serif text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Keep only restrained system feedback: status dots should blink briefly to suggest a live session, and list items should switch their background to #2A2520 on touch.
+- Button taps may use a subtle press effect; avoid bounce, rotation, or decorative motion. Keep all transitions fast, hard-edged, and industrial.
+# Layout
+- Use a dark, compact information flow, with a fixed 48px control bar at the top showing miniature navigation, issue tags, live status, and operator info.
+- The hero uses an oversized condensed title and a film still, with grayscale, contrast, and grain filters layered over the image, followed by a montage-style subtitle underneath.
+- Main content is arranged in dense cards, each module containing a large orange number, a short technical paragraph, and hairline separators. Side indexes become a vertical log list on mobile, with entries containing a timestamp, title, thumbnail block, and an "Enter" button.
+- All sections use square corners, no shadows, and low whitespace, with tightly joined borders to evoke an editing suite and render-farm console.
+# Elements
+- Cards, buttons, lists, and status panels all use square borders; rounded corners and shadows are forbidden.
+- Use crosshair markers, 1px coordinate lines, REC labels, timecodes, FPS, LUT, LOG-C, and other technical metadata to strengthen the post-production context.
+- Overlay subtle film noise on the background; images may use grayscale, low brightness, and high contrast filters to mimic old monitors and film projection.
+- Scrollbars, numbers, button outlines, and key status states all use #FF4500, while other information stays in warm bone white and gray-brown tiers.</t>
+        </is>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>Celluloid Noir</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>A dark film journal with the texture of an underground zine, blending an editing console, technical logs, film grain, and dense information layout. Cool, industrial, and tightly packed.</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W102" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t># Theme Name: Celluloid Noir
+# Vibe &amp; Description:
+A dark film journal with the texture of an underground zine, blending an editing console, technical logs, film grain, and dense information layout. Cool, industrial, and tightly packed.
+# Color
+- Keep colors strictly limited: deep caramel black, dark slate gray, warm bone white, gray-brown text, and electric orange.
+- Use #12100E for the background, #1A1714 / #1C1916 for modules, #D9D2C5 for text, and #A0988C for secondary information. Use only #FF4500 as the accent color for numbers, status dots, button borders, and thick dividers.
+- No pure white, pure black, bright backgrounds, or high-saturation colors other than orange. All dividers use 1px hairlines in #2C2824, and key areas may use 4px bars in #FF4500.
+# Font
+- Use "Muyao Softbrush" as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf)
+- Use "Source Han Serif CN" as the body, log, and metadata font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+# Animation
+- Keep only restrained system feedback: status dots should blink briefly to suggest a live session, and list items should switch their background to #2A2520 on touch.
+- Button taps may use a subtle press effect; avoid bounce, rotation, or decorative motion. Keep all transitions fast, hard-edged, and industrial.
+# Layout
+- Use a dark, compact information flow, with a fixed 48px control bar at the top showing miniature navigation, issue tags, live status, and operator info.
+- The hero uses an oversized condensed title and a film still, with grayscale, contrast, and grain filters layered over the image, followed by a montage-style subtitle underneath.
+- Main content is arranged in dense cards, each module containing a large orange number, a short technical paragraph, and hairline separators. Side indexes become a vertical log list on mobile, with entries containing a timestamp, title, thumbnail block, and an "Enter" button.
+- All sections use square corners, no shadows, and low whitespace, with tightly joined borders to evoke an editing suite and render-farm console.
+# Elements
+- Cards, buttons, lists, and status panels all use square borders; rounded corners and shadows are forbidden.
+- Use crosshair markers, 1px coordinate lines, REC labels, timecodes, FPS, LUT, LOG-C, and other technical metadata to strengthen the post-production context.
+- Overlay subtle film noise on the background; images may use grayscale, low brightness, and high contrast filters to mimic old monitors and film projection.
+- Scrollbars, numbers, button outlines, and key status states all use #FF4500, while other information stays in warm bone white and gray-brown tiers.</t>
+        </is>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>Quiet Luxury Retreat</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>Minimal luxury, Source Han Serif CN headlines, and warm-gold fine-line accents create a quiet, private, immersive resort atmosphere through generous whitespace, restrained typography, and high-quality hotel photography.</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W103" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t># Theme Name: Quiet Luxury Retreat
+# Vibe &amp; Description:
+Minimal luxury, Source Han Serif CN headlines, and warm-gold fine-line accents create a quiet, private, immersive resort atmosphere through generous whitespace, restrained typography, and high-quality hotel photography.
+# Color
+- Keep the palette restrained, using only deep navy, pure white, warm off-white, warm gold, and medium gray.
+- Backgrounds are mainly pure white (#FFFFFF) and warm off-white (#F8F7F4). Text uses deep navy (#1A1A2E), while secondary text uses medium gray (#888888). Warm gold (#C9A96E) is used only for ratings, badges, hover states, and fine details, conveying understated luxury.
+- CTAs may use near-black (#1A1A1A) with white text. Avoid gradients, highly saturated colors, and excessive decoration.
+# Font
+- Use "Source Han Serif CN" as the title font to create a refined, architectural-magazine feel. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use "Alibaba PuHuiTi" as the body font to maintain clarity, restraint, and modernity. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'SourceHanSerifCN-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the fontFamily property in `tailwind.config.js` to extend the fonts
+```js
+{
+  fontFamily: {
+    'title-serif-bold': ['SourceHanSerifCN-Bold', 'serif'],
+    'body-alibaba': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-serif-bold text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On card touch, slightly lift the card and enhance the shadow; on button tap, provide subtle scale feedback while keeping the motion quiet and restrained.
+- When page content appears, use fade-in with slight displacement. Statistics may count up after entering the viewport. Avoid flashy effects such as bouncing or rotation.
+# Layout
+- The page emphasizes generous whitespace and clear hierarchy, with large yet restrained titles and short body copy, resembling a high-end architecture and travel magazine.
+- In the mobile app, use a single-column immersive layout: establish the mood with a large hotel architecture photo at the top, then unfold through curated hotel cards, experience features, user reviews, and a subscription module.
+- Maintain ample spacing between cards. Let the interface recede as much as possible, allowing architectural photography, spatial light and shadow, and typographic hierarchy to take center stage.
+# Elements
+- Hotel cards use high-quality architectural photography, with a relatively vertical image ratio, moderate rounded corners, light default shadows, and a slight upward movement on touch.
+- Glass information cards can be overlaid on the Hero image, using translucent white, background blur, and an ultra-thin white border to create a private retreat feel.
+- Feature cards use an off-white background and large rounded corners, with concise icons, titles, and short descriptions.
+- Buttons use rounded pill shapes. Primary buttons use near-black backgrounds with white text, while subscription buttons may use white backgrounds with dark text. Use warm gold as the only accent color on hover or press.</t>
+        </is>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>Quiet Luxury Retreat</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>Minimal luxury, Source Han Serif CN headlines, and warm-gold fine-line accents create a quiet, private, immersive resort atmosphere through generous whitespace, restrained typography, and high-quality hotel photography.</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W104" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t># Theme Name: Quiet Luxury Retreat
+# Vibe &amp; Description:
+Minimal luxury, Source Han Serif CN headlines, and warm-gold fine-line accents create a quiet, private, immersive resort atmosphere through generous whitespace, restrained typography, and high-quality hotel photography.
+# Color
+- Keep the palette restrained, using only deep navy, pure white, warm off-white, warm gold, and medium gray.
+- Backgrounds are mainly pure white (#FFFFFF) and warm off-white (#F8F7F4). Text uses deep navy (#1A1A2E), while secondary text uses medium gray (#888888). Warm gold (#C9A96E) is used only for ratings, badges, hover states, and fine details, conveying understated luxury.
+- CTAs may use near-black (#1A1A1A) with white text. Avoid gradients, highly saturated colors, and excessive decoration.
+# Font
+- Use "Source Han Serif CN" as the title font to create a refined, architectural-magazine feel. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use "Alibaba PuHuiTi" as the body font to maintain clarity, restraint, and modernity. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- On card touch, slightly lift the card and enhance the shadow; on button tap, provide subtle scale feedback while keeping the motion quiet and restrained.
+- When page content appears, use fade-in with slight displacement. Statistics may count up after entering the viewport. Avoid flashy effects such as bouncing or rotation.
+# Layout
+- The page emphasizes generous whitespace and clear hierarchy, with large yet restrained titles and short body copy, resembling a high-end architecture and travel magazine.
+- In the mobile app, use a single-column immersive layout: establish the mood with a large hotel architecture photo at the top, then unfold through curated hotel cards, experience features, user reviews, and a subscription module.
+- Maintain ample spacing between cards. Let the interface recede as much as possible, allowing architectural photography, spatial light and shadow, and typographic hierarchy to take center stage.
+# Elements
+- Hotel cards use high-quality architectural photography, with a relatively vertical image ratio, moderate rounded corners, light default shadows, and a slight upward movement on touch.
+- Glass information cards can be overlaid on the Hero image, using translucent white, background blur, and an ultra-thin white border to create a private retreat feel.
+- Feature cards use an off-white background and large rounded corners, with concise icons, titles, and short descriptions.
+- Buttons use rounded pill shapes. Primary buttons use near-black backgrounds with white text, while subscription buttons may use white backgrounds with dark text. Use warm gold as the only accent color on hover or press.</t>
+        </is>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>Print Imperfect</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>Misregistered overprints, halftone dots, and a limited palette evoke the rough feel and handmade batch quality of old presses.</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W105" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t># Theme Name: Print Imperfect
+# Vibe &amp; Description:
+Misregistered overprints, halftone dots, and a limited palette evoke the rough feel and handmade batch quality of old presses.
+# Color
+- Keep colors tightly limited: use only paper white, coarse black, pink, and blue, with a small amount of orange for accents.
+- Use paper white (#FDFBF7) for the background, coarse black (#1A1A1A) for text and borders, print pink (#FF6B9D) for the primary color, and blue (#2563EB) for the secondary color. No gradients; all color blocks should stay flat, hard-edged, and direct.
+# Font
+- Use “YouSheBiaoTiHei” as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf)
+- Use “Alibaba PuHuiTi 3.0” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'YouSheBiaoTiHei-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the `fontFamily` property extension in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'title-youshe': ['YouSheBiaoTiHei-Regular', 'sans-serif'],
+    'body-alibaba': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-youshe text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- When a button or card is touched, the element shifts slightly down and right, and the hard shadow shrinks or disappears, simulating the feedback of pressed paper.
+- When elements appear, use a brief fade-in with misregistered overprint effects; slightly offset pink or blue shadows create the visual interest of imperfect registration.
+# Layout
+- Use a clear grid structure; cards, buttons, and navigation keep coarse black borders and hard-edge shadows, like a printed poster divided into sections.
+- On mobile, use a single-column layout with ample whitespace. Enlarge titles and set them in uppercase, monospace, bold typography to create a strong printed-heading feel.
+# Elements
+- Buttons and cards use `border-2 border-[#1A1A1A] rounded-sm`, paired with `shadow-[3px_3px_0px_#FF6B9D]` to create a hard-edged overprint shadow.
+- Overlay halftone-dot texture on parts of the background or cards, keeping low opacity to avoid affecting readability.
+- Use flat color blocks for icons, tags, and decorative blocks; avoid realistic lighting, blurred shadows, or complex gradients.
+- Accent text can use a subtle pink or blue offset outline to evoke the color-shift effect of print registration.</t>
+        </is>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>Print Imperfect</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>Misregistered overprints, halftone dots, and a limited palette evoke the rough feel and handmade batch quality of old presses.</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W106" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t># Theme Name: Print Imperfect
+# Vibe &amp; Description:
+Misregistered overprints, halftone dots, and a limited palette evoke the rough feel and handmade batch quality of old presses.
+# Color
+- Keep colors tightly limited: use only paper white, coarse black, pink, and blue, with a small amount of orange for accents.
+- Use paper white (#FDFBF7) for the background, coarse black (#1A1A1A) for text and borders, print pink (#FF6B9D) for the primary color, and blue (#2563EB) for the secondary color. No gradients; all color blocks should stay flat, hard-edged, and direct.
+# Font
+- Use “YouSheBiaoTiHei” as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf)
+- Use “Alibaba PuHuiTi 3.0” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- When a button or card is touched, the element shifts slightly down and right, and the hard shadow shrinks or disappears, simulating the feedback of pressed paper.
+- When elements appear, use a brief fade-in with misregistered overprint effects; slightly offset pink or blue shadows create the visual interest of imperfect registration.
+# Layout
+- Use a clear grid structure; cards, buttons, and navigation keep coarse black borders and hard-edge shadows, like a printed poster divided into sections.
+- On mobile, use a single-column layout with ample whitespace. Enlarge titles and set them in uppercase, monospace, bold typography to create a strong printed-heading feel.
+# Elements
+- Buttons and cards use `border-2 border-[#1A1A1A] rounded-sm`, paired with `shadow-[3px_3px_0px_#FF6B9D]` to create a hard-edged overprint shadow.
+- Overlay halftone-dot texture on parts of the background or cards, keeping low opacity to avoid affecting readability.
+- Use flat color blocks for icons, tags, and decorative blocks; avoid realistic lighting, blurred shadows, or complex gradients.
+- Accent text can use a subtle pink or blue offset outline to evoke the color-shift effect of print registration.</t>
+        </is>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>Pixel Arcade</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>Retro 8-bit game visuals, hard-edged outlines, high-saturation pixel colors, emphasizing no rounded corners, thick borders, and instant feedback, evoking classic arcade and indie-game nostalgia.</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W107" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t># Theme Name: Pixel Arcade
+# Vibe &amp; Description:
+Retro 8-bit game visuals, hard-edged outlines, high-saturation pixel colors, emphasizing no rounded corners, thick borders, and instant feedback, evoking classic arcade and indie-game nostalgia.
+# Color
+- Use a classic 8-bit palette; avoid gradients, alpha transitions, and soft colors.
+- Use dark pixel black (#1A1C2C) for backgrounds and borders, bright white (#F4F4F4) for base backgrounds, and red (#FF004D), green (#00E436), blue (#29ADFF), and yellow (#FFEC27) for accents. The overall palette should be direct, vivid, and high-contrast, as clear and forceful as an early game interface.
+# Font
+- Use “ChillBitmap 16px” as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/ChillBitmap_16px.ttf)
+- Use “Alibaba PuHuiTi” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'ChillBitmap-16px': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/ChillBitmap_16px.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the `fontFamily` property to `tailwind.config.js` to extend the fonts
+```js
+{
+  fontFamily: {
+    'title-hanchandianzhen': ['ChillBitmap-16px', 'monospace'],
+    'body-alibaba': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-hanchandianzhen text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- All interactions use instant hard cuts, with no easing, gradients, or opacity animations. On touch, elements move 1-2px down and to the right while the shadow shortens or disappears, creating feedback like a pressed physical button.
+- Hover or selected states use Palette Swap, switching directly to another 8-bit accent color, such as a red button turning blue, with no intermediate transition.
+# Layout
+- Keep the page structure clearly segmented, using thick borders and hard-edged shadows to create hierarchy. Cards, buttons, and input fields should all stay square, with no rounded corners.
+- In a mobile app, keep the grid compact but rhythmic, with clear spacing between modules. Key areas can use yellow headings, red action buttons, and blue-green status accents.
+# Elements
+- Use `border-4`, `rounded-none`, and `shadow-[4px_4px_0_#1a1c2c]` for buttons; shift them and remove the shadow on click.
+- Cards use a white background, dark thick borders, and hard shadows, staying stable and clear like a game menu panel.
+- Input fields keep a square outline; on focus, use a blue inner outline, with no glow or soft shadow.
+- Decorative elements may include pixel stars, blocks, health bars, leaderboard items, and similar graphics, but keep them restrained to avoid weakening readability.</t>
+        </is>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>Pixel Arcade</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>Retro 8-bit game visuals, hard-edged outlines, high-saturation pixel colors, emphasizing no rounded corners, thick borders, and instant feedback, evoking classic arcade and indie-game nostalgia.</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W108" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t># Theme Name: Pixel Arcade
+# Vibe &amp; Description:
+Retro 8-bit game visuals, hard-edged outlines, high-saturation pixel colors, emphasizing no rounded corners, thick borders, and instant feedback, evoking classic arcade and indie-game nostalgia.
+# Color
+- Use a classic 8-bit palette; avoid gradients, alpha transitions, and soft colors.
+- Use dark pixel black (#1A1C2C) for backgrounds and borders, bright white (#F4F4F4) for base backgrounds, and red (#FF004D), green (#00E436), blue (#29ADFF), and yellow (#FFEC27) for accents. The overall palette should be direct, vivid, and high-contrast, as clear and forceful as an early game interface.
+# Font
+- Use “ChillBitmap 16px” as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/ChillBitmap_16px.ttf)
+- Use “Alibaba PuHuiTi” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- All interactions use instant hard cuts, with no easing, gradients, or opacity animations. On touch, elements move 1-2px down and to the right while the shadow shortens or disappears, creating feedback like a pressed physical button.
+- Hover or selected states use Palette Swap, switching directly to another 8-bit accent color, such as a red button turning blue, with no intermediate transition.
+# Layout
+- Keep the page structure clearly segmented, using thick borders and hard-edged shadows to create hierarchy. Cards, buttons, and input fields should all stay square, with no rounded corners.
+- In a mobile app, keep the grid compact but rhythmic, with clear spacing between modules. Key areas can use yellow headings, red action buttons, and blue-green status accents.
+# Elements
+- Use `border-4`, `rounded-none`, and `shadow-[4px_4px_0_#1a1c2c]` for buttons; shift them and remove the shadow on click.
+- Cards use a white background, dark thick borders, and hard shadows, staying stable and clear like a game menu panel.
+- Input fields keep a square outline; on focus, use a blue inner outline, with no glow or soft shadow.
+- Decorative elements may include pixel stars, blocks, health bars, leaderboard items, and similar graphics, but keep them restrained to avoid weakening readability.</t>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>Watercolor Wash</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>Soft gradients, paper texture, and layered translucent color washes emphasize fluidity, poetry, and artistry, evoking the visual experience of watercolor naturally spreading across paper.</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W109" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t># Theme Name: Watercolor Wash
+# Vibe &amp; Description:
+Soft gradients, paper texture, and layered translucent color washes emphasize fluidity, poetry, and artistry, evoking the visual experience of watercolor naturally spreading across paper.
+# Color
+- Use warm paper tone `#FAF8F5` for the background, avoiding pure white that feels too cold or pure black that feels too harsh.
+- Use calm blue `#4A6FA5` as the primary color, paired with low-saturation watercolor accents: terracotta orange `#E8A87C`, lake cyan `#85CDCA`, rose gray `#C38D94`, and warm brown `#D4A373`.
+- Use translucent gradients for cards and overlays, such as `from-white/70 to-[#4A6FA5]/10`, to create a layered watercolor effect.
+- Use extremely pale blue-gray borders: `border-[#4A6FA5]/20`. Avoid hard black borders, pure black backgrounds, and high-contrast rigid dividers.
+# Font
+- Use “MuyaoSoftbrush” as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf)
+- Use “ResourceHanRoundedCN” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'MuyaoSoftbrush-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf' },
+  'ResourceHanRoundedCN-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Regular.ttf' },
+});
+```
+Add the fontFamily extension to `tailwind.config.js`
+```js
+{
+  fontFamily: {
+   'title-muyao': ['MuyaoSoftbrush-Regular', 'sans-serif'],
+   'body-resource-rounded': ['ResourceHanRoundedCN-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-muyao text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-resource-rounded text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch, elements scale up slightly, such as `scale(1.02)`, and shrink back slightly when pressed, such as `scale(0.98)`, avoiding rigid displacement.
+- When elements appear, use soft fade-ins, slight blur diffusion, or layered opacity, like watercolor pigment gradually seeping into paper.
+- Keep transitions slow and natural; `duration-400 ease-out` is recommended.
+# Layout
+- Preserve generous whitespace on the page, like content layers unfolding naturally on drawing paper.
+- Cards use large rounded corners and softened shadows; `rounded-2xl` or `rounded-3xl` is recommended. Avoid sharp corners and strong drop shadows.
+- Establish content hierarchy through font size, opacity, color depth, and whitespace, rather than relying on heavy divider lines.
+# Elements
+- Overlay soft watercolor gradient patches on the background; use low opacity, blur, and irregular positioning to create a sense of pigment diffusion.
+- Buttons use pill shapes or large rounded rectangles, paired with translucent fills and soft shadows.
+- Cards use translucent gradient backgrounds, thin borders, and light shadows to keep edges soft.
+- Decorative elements may include pale water stains, paper noise, hand-drawn lines, or blurred color blocks, while keeping the overall style restrained, quiet, and translucent.</t>
+        </is>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Watercolor Wash</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>Soft gradients, paper texture, and layered translucent color washes emphasize fluidity, poetry, and artistry, evoking the visual experience of watercolor naturally spreading across paper.</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W110" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y110" t="inlineStr">
+        <is>
+          <t># Theme Name: Watercolor Wash
+# Vibe &amp; Description:
+Soft gradients, paper texture, and layered translucent color washes emphasize fluidity, poetry, and artistry, evoking the visual experience of watercolor naturally spreading across paper.
+# Color
+- Use warm paper tone `#FAF8F5` for the background, avoiding pure white that feels too cold or pure black that feels too harsh.
+- Use calm blue `#4A6FA5` as the primary color, paired with low-saturation watercolor accents: terracotta orange `#E8A87C`, lake cyan `#85CDCA`, rose gray `#C38D94`, and warm brown `#D4A373`.
+- Use translucent gradients for cards and overlays, such as `from-white/70 to-[#4A6FA5]/10`, to create a layered watercolor effect.
+- Use extremely pale blue-gray borders: `border-[#4A6FA5]/20`. Avoid hard black borders, pure black backgrounds, and high-contrast rigid dividers.
+# Font
+- Use “MuyaoSoftbrush” as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf)
+- Use “ResourceHanRoundedCN” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Regular.ttf)
+# Animation
+- On touch, elements scale up slightly, such as `scale(1.02)`, and shrink back slightly when pressed, such as `scale(0.98)`, avoiding rigid displacement.
+- When elements appear, use soft fade-ins, slight blur diffusion, or layered opacity, like watercolor pigment gradually seeping into paper.
+- Keep transitions slow and natural; `duration-400 ease-out` is recommended.
+# Layout
+- Preserve generous whitespace on the page, like content layers unfolding naturally on drawing paper.
+- Cards use large rounded corners and softened shadows; `rounded-2xl` or `rounded-3xl` is recommended. Avoid sharp corners and strong drop shadows.
+- Establish content hierarchy through font size, opacity, color depth, and whitespace, rather than relying on heavy divider lines.
+# Elements
+- Overlay soft watercolor gradient patches on the background; use low opacity, blur, and irregular positioning to create a sense of pigment diffusion.
+- Buttons use pill shapes or large rounded rectangles, paired with translucent fills and soft shadows.
+- Cards use translucent gradient backgrounds, thin borders, and light shadows to keep edges soft.
+- Decorative elements may include pale water stains, paper noise, hand-drawn lines, or blurred color blocks, while keeping the overall style restrained, quiet, and translucent.</t>
+        </is>
+      </c>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>Ink Wash Reverie</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>Sparse ink and xuan paper texture blend calligraphy, distant mountains, seals, and diffused ink washes to create a serene, deep, poetic Eastern atmosphere.</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W111" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y111" t="inlineStr">
+        <is>
+          <t># Theme Name: Ink Wash Reverie
+# Vibe &amp; Description:
+Sparse ink and xuan paper texture blend calligraphy, distant mountains, seals, and diffused ink washes to create a serene, deep, poetic Eastern atmosphere.
+# Color
+- Center on xuan paper white and layered ink tones, strictly avoiding neon colors, highly saturated colors, and large areas of pure black backgrounds.
+- Use xuan paper white (#F8F5F0), beige (#FAF0E6), or ivory white (#FFFFF0) for backgrounds, and burnt ink (#1A1A1A), deep ink (#333333), light ink (#666666), and pale ink (#999999) for text.
+- Keep accent colors restrained: vermilion seal red (#C41E3A) for seals and key markers, verdant landscape green (#2E8B57) for very small amounts of mountain-and-water imagery, and gold (#D4AF37) only for premium decorative details.
+# Font
+- Use "AlimamaDongFangDaKai" as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/AlimamaDongFangDaKai-Regular.ttf)
+- Use "SourceHanSerifCN" as the subtitle and navigation font, preserving a smooth, upright handwritten feel. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'AlimamaDongFangDaKai-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlimamaDongFangDaKai-Regular.ttf' },
+  'SourceHanSerifCN-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2' },
+});
+```
+Add a fontFamily property to `tailwind.config.js` to extend the fonts
+```js
+{
+  fontFamily: {
+    'title-dongfangdakai': ['AlimamaDongFangDaKai-Regular', 'serif'],
+    'body-serif': ['SourceHanSerifCN-Regular', 'serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-dongfangdakai text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-serif text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch or long press, elements produce a slight ink diffusion, with softened edges and changing opacity, like ink slowly soaking into xuan paper.
+- When page elements appear, use a "fade in + slight rise" or "mist gradually emerging" transition, with a duration of 300-500ms, keeping the pace subtle, slow, and poetic.
+# Layout
+- Leave ample white space on the page, with elements distributed loosely to avoid crowding and rigid geometric order.
+- The composition can be slightly asymmetrical to form a natural landscape painting feel; titles may be larger, body text restrained, and vertical decorative text can be added locally to enhance the classical mood.
+- In mobile apps, use a mainly single-column layout, preserving calligraphy titles, xuan paper backgrounds, and white-space rhythm, with touch targets no smaller than 44px.
+# Elements
+- Cards and buttons use soft ink-toned edges, avoiding hard-edged shadows; blur, translucency, and irregular shapes can be used to mimic brushstrokes.
+- Seals serve as key visual symbols, using vermilion square or circular shapes, with small accents on titles, buttons, or blank areas.
+- Overlay the background with subtle xuan paper grain texture, and add abstract distant mountains, bamboo, plum, orchid, and chrysanthemum line art, or light ink splashes as decoration.
+- Dividers and decorative shapes should feel dry-brushed, diffused, or balanced between solid and void, avoiding modern industrial icons and sharp geometric borders.</t>
+        </is>
+      </c>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>Ink Wash Reverie</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>Sparse ink and xuan paper texture blend calligraphy, distant mountains, seals, and diffused ink washes to create a serene, deep, poetic Eastern atmosphere.</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W112" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t># Theme Name: Ink Wash Reverie
+# Vibe &amp; Description:
+Sparse ink and xuan paper texture blend calligraphy, distant mountains, seals, and diffused ink washes to create a serene, deep, poetic Eastern atmosphere.
+# Color
+- Center on xuan paper white and layered ink tones, strictly avoiding neon colors, highly saturated colors, and large areas of pure black backgrounds.
+- Use xuan paper white (#F8F5F0), beige (#FAF0E6), or ivory white (#FFFFF0) for backgrounds, and burnt ink (#1A1A1A), deep ink (#333333), light ink (#666666), and pale ink (#999999) for text.
+- Keep accent colors restrained: vermilion seal red (#C41E3A) for seals and key markers, verdant landscape green (#2E8B57) for very small amounts of mountain-and-water imagery, and gold (#D4AF37) only for premium decorative details.
+# Font
+- Use "AlimamaDongFangDaKai" as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/AlimamaDongFangDaKai-Regular.ttf)
+- Use "SourceHanSerifCN" as the subtitle and navigation font, preserving a smooth, upright handwritten feel. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+# Animation
+- On touch or long press, elements produce a slight ink diffusion, with softened edges and changing opacity, like ink slowly soaking into xuan paper.
+- When page elements appear, use a "fade in + slight rise" or "mist gradually emerging" transition, with a duration of 300-500ms, keeping the pace subtle, slow, and poetic.
+# Layout
+- Leave ample white space on the page, with elements distributed loosely to avoid crowding and rigid geometric order.
+- The composition can be slightly asymmetrical to form a natural landscape painting feel; titles may be larger, body text restrained, and vertical decorative text can be added locally to enhance the classical mood.
+- In mobile apps, use a mainly single-column layout, preserving calligraphy titles, xuan paper backgrounds, and white-space rhythm, with touch targets no smaller than 44px.
+# Elements
+- Cards and buttons use soft ink-toned edges, avoiding hard-edged shadows; blur, translucency, and irregular shapes can be used to mimic brushstrokes.
+- Seals serve as key visual symbols, using vermilion square or circular shapes, with small accents on titles, buttons, or blank areas.
+- Overlay the background with subtle xuan paper grain texture, and add abstract distant mountains, bamboo, plum, orchid, and chrysanthemum line art, or light ink splashes as decoration.
+- Dividers and decorative shapes should feel dry-brushed, diffused, or balanced between solid and void, avoiding modern industrial icons and sharp geometric borders.</t>
+        </is>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>Coral Beat</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>A light music player style, where a warm ivory background and pure white cards create a soothing, translucent atmosphere. Coral orange accents the playback controls, making the overall feel soft, modern, airy, and rhythmic.</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W113" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t># Theme Name: Coral Beat
+# Vibe &amp; Description:
+A light music player style, where a warm ivory background and pure white cards create a soothing, translucent atmosphere. Coral orange accents the playback controls, making the overall feel soft, modern, airy, and rhythmic.
+# Color
+- Use a warm light color system, avoiding dark backgrounds and highly saturated neon colors.
+- Use warm ivory (#F8F6F2) for the background, pure white (#FFFFFF) for cards, menus, and the bottom playback bar, dark gray-black (#1C1C1E) for text, and soft gray (#6C6C70) for secondary text.
+- Use coral orange (#F97316) as the accent color, mainly for play buttons, progress states, and key interaction feedback. Use light gray (#EBEBEB / #EFEFEF) for dividers to keep the interface clean and airy.
+# Font
+- Use the title font “YouSheBiaoTiHei” for song names with a medium-bold weight, creating a clear but not heavy hierarchy for music cards.（https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf）
+- Use the body font “ResourceHanRoundedCN” for menu items in regular weight, while supporting information such as artist names and durations uses a lighter gray and smaller font size.（https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Regular.ttf）
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'YouSheBiaoTiHei-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf' },
+  'ResourceHanRoundedCN-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Regular.ttf' },
+});
+```
+Add the fontFamily extension in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'title-youshe': ['YouSheBiaoTiHei-Regular', 'sans-serif'],
+    'body-resource-rounded': ['ResourceHanRoundedCN-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-youshe text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-resource-rounded text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch, cards rise slightly and deepen their shadow, simulating a light selected-state response for playlists.
+- When tapped or hovered, the play button scales up to 1.05, emphasizing the immediacy of music controls.
+- Menu item switching uses short transitions, with the highlight background changing from transparent to a light gray rounded block to stay soft and natural.
+- On touch, the progress bar shifts from light gray to brighter color to indicate interactivity, but real audio dragging is not required.
+# Layout
+- The mobile app uses a single-column main content layout, with a warm ivory overall background and around 16px padding in the content area.
+- The top displays a greeting and lightweight status entry, followed by a “Now Playing” mini card containing cover art, song name, artist, a simple progress bar, and playback controls.
+- Recommended playlists use a single-column card feed, with each card containing a light gradient cover placeholder, title, and artist information.
+- The recently played list uses a compact row layout, showing index number, song name, artist, and duration, with light gray dividers between rows.
+- The fixed bottom playback bar is about 80px high and includes the current song thumbnail, song information, play button, and simplified progress state.
+# Elements
+- Cards consistently use a pure white background, 16px rounded corners, and a light shadow, avoiding heavy shadows and overly large corner radii.
+- Cover placeholders may use soft light gradients and music icons as the only permitted subtle gradient element.
+- The play button uses a coral orange circular or emphasized style, while previous and next buttons remain dark gray linear icons.
+- Menu highlights use a light gray rounded background, without strong color blocks.
+- The bottom playback bar uses a pure white background with a light gray top divider, forming a stable player anchor.</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Coral Beat</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>A light music player style, where a warm ivory background and pure white cards create a soothing, translucent atmosphere. Coral orange accents the playback controls, making the overall feel soft, modern, airy, and rhythmic.</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W114" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t># Theme Name: Coral Beat
+# Vibe &amp; Description:
+A light music player style, where a warm ivory background and pure white cards create a soothing, translucent atmosphere. Coral orange accents the playback controls, making the overall feel soft, modern, airy, and rhythmic.
+# Color
+- Use a warm light color system, avoiding dark backgrounds and highly saturated neon colors.
+- Use warm ivory (#F8F6F2) for the background, pure white (#FFFFFF) for cards, menus, and the bottom playback bar, dark gray-black (#1C1C1E) for text, and soft gray (#6C6C70) for secondary text.
+- Use coral orange (#F97316) as the accent color, mainly for play buttons, progress states, and key interaction feedback. Use light gray (#EBEBEB / #EFEFEF) for dividers to keep the interface clean and airy.
+# Font
+- Use the title font “YouSheBiaoTiHei” for song names with a medium-bold weight, creating a clear but not heavy hierarchy for music cards.（https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf）
+- Use the body font “ResourceHanRoundedCN” for menu items in regular weight, while supporting information such as artist names and durations uses a lighter gray and smaller font size.（https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Regular.ttf）
+# Animation
+- On touch, cards rise slightly and deepen their shadow, simulating a light selected-state response for playlists.
+- When tapped or hovered, the play button scales up to 1.05, emphasizing the immediacy of music controls.
+- Menu item switching uses short transitions, with the highlight background changing from transparent to a light gray rounded block to stay soft and natural.
+- On touch, the progress bar shifts from light gray to brighter color to indicate interactivity, but real audio dragging is not required.
+# Layout
+- The mobile app uses a single-column main content layout, with a warm ivory overall background and around 16px padding in the content area.
+- The top displays a greeting and lightweight status entry, followed by a “Now Playing” mini card containing cover art, song name, artist, a simple progress bar, and playback controls.
+- Recommended playlists use a single-column card feed, with each card containing a light gradient cover placeholder, title, and artist information.
+- The recently played list uses a compact row layout, showing index number, song name, artist, and duration, with light gray dividers between rows.
+- The fixed bottom playback bar is about 80px high and includes the current song thumbnail, song information, play button, and simplified progress state.
+# Elements
+- Cards consistently use a pure white background, 16px rounded corners, and a light shadow, avoiding heavy shadows and overly large corner radii.
+- Cover placeholders may use soft light gradients and music icons as the only permitted subtle gradient element.
+- The play button uses a coral orange circular or emphasized style, while previous and next buttons remain dark gray linear icons.
+- Menu highlights use a light gray rounded background, without strong color blocks.
+- The bottom playback bar uses a pure white background with a light gray top divider, forming a stable player anchor.</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>Glitch Canvas</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Cyberpunk glitch art: neon on black, a high-tech low-life dystopian atmosphere. Scan lines, chromatic offsets, beveled edges, and terminal-code aesthetics form a dangerous, rebellious, mechanized visual language.</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W115" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t># Theme Name: Glitch Canvas
+# Vibe &amp; Description:
+Cyberpunk glitch art: neon on black, a high-tech low-life dystopian atmosphere. Scan lines, chromatic offsets, beveled edges, and terminal-code aesthetics form a dangerous, rebellious, mechanized visual language.
+# Color
+- Use near-black with a purple undertone as the primary background, avoiding any light mode. Background color is #0A0A0F, card color is #12121A, and border color is #2A2A3A.
+- Highlights center on neon green #00FF88 for buttons, cursors, and key borders; magenta #FF00FF and cyan-blue #00D4FF are used for glitch offsets, auxiliary glow, and scan textures. Body text uses #E0E0E0, secondary text uses #6B7280, and danger alerts use #FF3366.
+# Font
+- Use “GlowSansSC-Normal-Bold” as the title font to maintain a mechanical, futuristic, wide-tracked visual feel. (https://resource-static.bj.bcebos.com/fonts-skill/GlowSansSC-Normal-Bold.woff2)
+- Use “AlibabaPuHuiTi-Regular” as the body, terminal, and label font to reinforce the code interface and hacker-terminal atmosphere. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'GlowSansSC-Normal-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/GlowSansSC-Normal-Bold.woff2' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the fontFamily extension in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'title-future': ['GlowSansSC-Normal-Bold', 'sans-serif'],
+    'body-alibaba': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-future text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Trigger short mechanical feedback on touch: slight displacement, flicker, and intensified neon glow. Avoid soft easing; use a linear or step rhythm.
+- Titles and key text may include red-blue chromatic offsets and subtle glitch jitter; terminal areas use cursor blinking, flowing scan lines, and typewriter-style reveal effects.
+# Layout
+- Use a dark full-screen background overlaid with scan lines, noise, and circuit textures. Content follows an 8px spacing grid; cards may use asymmetrical arrangements to create a sliced, misaligned futuristic interface feel.
+- On mobile, prioritize a single-column layout, with touch targets no smaller than 44px. Reduce excessive glow while preserving the core identity of black backgrounds, neon, terminals, and glitch textures.
+# Elements
+- Buttons and cards must not use rounded corners; use sharp corners, beveled corners, or SVG / Skia clipped shapes, with borders stroked in neon green or dark purple-gray.
+- Titles use RGB chromatic shadows, cards use neon box-shadow, and dividers use scan-line or circuit-line patterns.
+- Keep at least one terminal command-line module containing `$`, `&gt;_`, green code text, and a blinking cursor.
+- Overlay the background with a repeating-linear-gradient scan texture, adding localized magenta and cyan-blue glows to create an aged monitor glitch effect.</t>
+        </is>
+      </c>
+      <c r="Z115" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>Glitch Canvas</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>Cyberpunk glitch art: neon on black, a high-tech low-life dystopian atmosphere. Scan lines, chromatic offsets, beveled edges, and terminal-code aesthetics form a dangerous, rebellious, mechanized visual language.</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W116" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y116" t="inlineStr">
+        <is>
+          <t># Theme Name: Glitch Canvas
+# Vibe &amp; Description:
+Cyberpunk glitch art: neon on black, a high-tech low-life dystopian atmosphere. Scan lines, chromatic offsets, beveled edges, and terminal-code aesthetics form a dangerous, rebellious, mechanized visual language.
+# Color
+- Use near-black with a purple undertone as the primary background, avoiding any light mode. Background color is #0A0A0F, card color is #12121A, and border color is #2A2A3A.
+- Highlights center on neon green #00FF88 for buttons, cursors, and key borders; magenta #FF00FF and cyan-blue #00D4FF are used for glitch offsets, auxiliary glow, and scan textures. Body text uses #E0E0E0, secondary text uses #6B7280, and danger alerts use #FF3366.
+# Font
+- Use “GlowSansSC-Normal-Bold” as the title font to maintain a mechanical, futuristic, wide-tracked visual feel. (https://resource-static.bj.bcebos.com/fonts-skill/GlowSansSC-Normal-Bold.woff2)
+- Use “AlibabaPuHuiTi-Regular” as the body, terminal, and label font to reinforce the code interface and hacker-terminal atmosphere. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- Trigger short mechanical feedback on touch: slight displacement, flicker, and intensified neon glow. Avoid soft easing; use a linear or step rhythm.
+- Titles and key text may include red-blue chromatic offsets and subtle glitch jitter; terminal areas use cursor blinking, flowing scan lines, and typewriter-style reveal effects.
+# Layout
+- Use a dark full-screen background overlaid with scan lines, noise, and circuit textures. Content follows an 8px spacing grid; cards may use asymmetrical arrangements to create a sliced, misaligned futuristic interface feel.
+- On mobile, prioritize a single-column layout, with touch targets no smaller than 44px. Reduce excessive glow while preserving the core identity of black backgrounds, neon, terminals, and glitch textures.
+# Elements
+- Buttons and cards must not use rounded corners; use sharp corners, beveled corners, or SVG / Skia clipped shapes, with borders stroked in neon green or dark purple-gray.
+- Titles use RGB chromatic shadows, cards use neon box-shadow, and dividers use scan-line or circuit-line patterns.
+- Keep at least one terminal command-line module containing `$`, `&gt;_`, green code text, and a blinking cursor.
+- Overlay the background with a repeating-linear-gradient scan texture, adding localized magenta and cyan-blue glows to create an aged monitor glitch effect.</t>
+        </is>
+      </c>
+      <c r="Z116" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Pink Noir Gallery</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>Deep black backdrop, high-saturation pink accents, a minimalist magazine-style gallery layout, and a calm, sharp editorial art-book presence.</t>
+        </is>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W117" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y117" t="inlineStr">
+        <is>
+          <t># Theme Name: Pink Noir Gallery
+# Vibe &amp; Description:
+Deep black backdrop, high-saturation pink accents, a minimalist magazine-style gallery layout, and a calm, sharp editorial art-book presence.
+# Color
+- Use deep black as the main background, paired with dark gray-black cards and high-saturation pink accents.
+- Background uses #121212, cards use #1C1C1C, and text is mainly high-contrast white and light gray. The accent color uses HSL(340, 80%, 62%) for buttons, selected states, glows, tags, and key interaction feedback, creating a strong yet restrained visual impact.
+# Font
+- Title: HarmonyOS Sans (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Bold.ttf)
+- Body: HarmonyOS Sans (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+## Font Import Method
+Use system fonts in `app/_layout.tsx`; no extra font files need to be loaded.
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'HarmonyOSSans-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Bold.ttf' },
+  'HarmonyOSSans-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf' },
+});
+```
+`tailwind.config.js` can keep the default `fontFamily`, or extend the system font family.
+```js
+{
+  fontFamily: {
+   'harmony-title': ['HarmonyOSSans-Bold', 'sans-serif'],
+    'harmony-body': ['HarmonyOSSans-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-harmony-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-harmony-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Cards lift slightly on touch, with deeper shadows to create a refined gallery hover feel. Button taps use a brief opacity or scale response, avoiding flashy motion.
+- When an image opens, use a dark overlay and a subtle scale-in effect, simulating an immersive preview as the work is placed under a spotlight. Mode switching, layout switching, and content reveal should keep a smooth 0.2-0.25s transition.
+# Layout
+- On mobile, use a single-column or two-column portfolio flow, with generous spacing between cards for an open, restrained feel, like a dark art portfolio.
+- The home screen emphasizes a large title, short description, and primary action button. The works area supports grid, magazine-style offset layout, and masonry-style arrangement. Editing controls appear only when needed and do not cover the main work.
+# Elements
+- Cards use 12px rounded corners, images use 8px rounded corners, and buttons use pill-shaped corners, keeping the overall edges soft but not overly rounded.
+- Artwork images support tap-to-zoom, with a darkened background, and the close button and action controls use pink accents.
+- Tags, layout toggle buttons, and edit entry points use subtle highlights, keeping functions clear without breaking the gallery atmosphere.
+- Heavy shadows, complex textures, large gradients, and fixed-width layouts are forbidden; keep it minimalist, responsive, and high-contrast.</t>
+        </is>
+      </c>
+      <c r="Z117" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>Pink Noir Gallery</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>Deep black backdrop, high-saturation pink accents, a minimalist magazine-style gallery layout, and a calm, sharp editorial art-book presence.</t>
+        </is>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W118" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y118" t="inlineStr">
+        <is>
+          <t># Theme Name: Pink Noir Gallery
+# Vibe &amp; Description:
+Deep black backdrop, high-saturation pink accents, a minimalist magazine-style gallery layout, and a calm, sharp editorial art-book presence.
+# Color
+- Use deep black as the main background, paired with dark gray-black cards and high-saturation pink accents.
+- Background uses #121212, cards use #1C1C1C, and text is mainly high-contrast white and light gray. The accent color uses HSL(340, 80%, 62%) for buttons, selected states, glows, tags, and key interaction feedback, creating a strong yet restrained visual impact.
+# Font
+- Title: HarmonyOS Sans (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Bold.ttf)
+- Body: HarmonyOS Sans (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+# Animation
+- Cards lift slightly on touch, with deeper shadows to create a refined gallery hover feel. Button taps use a brief opacity or scale response, avoiding flashy motion.
+- When an image opens, use a dark overlay and a subtle scale-in effect, simulating an immersive preview as the work is placed under a spotlight. Mode switching, layout switching, and content reveal should keep a smooth 0.2-0.25s transition.
+# Layout
+- On mobile, use a single-column or two-column portfolio flow, with generous spacing between cards for an open, restrained feel, like a dark art portfolio.
+- The home screen emphasizes a large title, short description, and primary action button. The works area supports grid, magazine-style offset layout, and masonry-style arrangement. Editing controls appear only when needed and do not cover the main work.
+# Elements
+- Cards use 12px rounded corners, images use 8px rounded corners, and buttons use pill-shaped corners, keeping the overall edges soft but not overly rounded.
+- Artwork images support tap-to-zoom, with a darkened background, and the close button and action controls use pink accents.
+- Tags, layout toggle buttons, and edit entry points use subtle highlights, keeping functions clear without breaking the gallery atmosphere.
+- Heavy shadows, complex textures, large gradients, and fixed-width layouts are forbidden; keep it minimalist, responsive, and high-contrast.</t>
+        </is>
+      </c>
+      <c r="Z118" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>Wabi-Sabi Verdure</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Eastern minimalism, wabi-sabi negative space, natural textures, with deep bamboo green and warm white tones, highlighting the vitality of plants, the warmth of handmade craft, and a quiet, lived-in atmosphere.</t>
+        </is>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W119" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y119" t="inlineStr">
+        <is>
+          <t># Theme Name: Wabi-Sabi Verdure
+# Vibe &amp; Description:
+Eastern minimalism, wabi-sabi negative space, natural textures, with deep bamboo green and warm white tones, highlighting the vitality of plants, the warmth of handmade craft, and a quiet, lived-in atmosphere.
+# Color
+- Use warm white (#FAFAF7) as the main background, creating natural whitespace and a soft paper feel.
+- Deep bamboo green (#2D5016) as the primary color, for navigation, buttons, prices, and key actions.
+- Charcoal gray (#2C2C2C) for body copy and explanatory text, keeping it clear without feeling harsh.
+- Pale gold (#C9A84C) only as a subtle accent, for tags, thin lines, price emphasis, or decorative gold lines.
+- Dark areas can use light bamboo green (#1E3A0F) with warm white text to create calm brand sections.
+# Font
+- Use "SourceHanSerifCN" for brand titles, page titles, and key numerals. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-SemiBold.woff2)
+- Use "SourceHanSerifCN" for body text, navigation, buttons, and explanatory copy. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+## Font Import Method
+Load the font in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'SourceHanSerifCN-SemiBold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-SemiBold.woff2' },
+  'SourceHanSerifCN-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2' },
+});
+```
+Add the `fontFamily` property in `tailwind.config.js` to extend the font set
+```js
+{
+  fontFamily: {
+    'source-serif-title': ['SourceHanSerifCN-SemiBold', 'serif'],
+    'source-serif-body': ['SourceHanSerifCN-Regular', 'serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-source-serif-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-source-serif-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Use a subtle 160ms press feedback on button tap, keeping it restrained, quick, and natural.
+- For cards, products, and image-text sections, use a "fade in + slide up" entrance animation, with staggered delays to create a quiet sense of ritual.
+- On hover or touch, cards rise slightly by 2px, with softly enhanced borders or shadows, avoiding exaggerated motion.
+- Respect `prefers-reduced-motion` by disabling transitions and entrance animations when motion is reduced.
+# Layout
+- The page should scroll vertically, with ample whitespace and clear section breaks.
+- Use an asymmetrical relationship between content and imagery, echoing a 60% information and 40% visual balance.
+- Spacing follows a 4px grid, with generous breathing room between paragraphs, compact heading line height, and loose body line height.
+- Product cards, brand intro sections, and cart areas should be grouped softly to avoid dense stacking.
+# Elements
+- Buttons use 8px corner radius, cards use 12px-16px corner radius, avoiding an overly cute fully rounded look.
+- Tags use a pale gold background and small rounded corners to present lightweight information such as "Best Seller" and "New".
+- Borders use semi-transparent deep bamboo green or charcoal gray, and cards have no heavy default shadow, keeping the look flat and quiet.
+- Dividers can use a bamboo-stem gradient line or a 1px pale gold line as a refined Eastern detail.
+- Choose low-saturation plant photography, emphasizing natural textures, soil, leaves, and light and shadow, without cluttered backgrounds.</t>
+        </is>
+      </c>
+      <c r="Z119" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>Wabi-Sabi Verdure</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>Eastern minimalism, wabi-sabi negative space, natural textures, with deep bamboo green and warm white tones, highlighting the vitality of plants, the warmth of handmade craft, and a quiet, lived-in atmosphere.</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W120" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y120" t="inlineStr">
+        <is>
+          <t># Theme Name: Wabi-Sabi Verdure
+# Vibe &amp; Description:
+Eastern minimalism, wabi-sabi negative space, natural textures, with deep bamboo green and warm white tones, highlighting the vitality of plants, the warmth of handmade craft, and a quiet, lived-in atmosphere.
+# Color
+- Use warm white (#FAFAF7) as the main background, creating natural whitespace and a soft paper feel.
+- Deep bamboo green (#2D5016) as the primary color, for navigation, buttons, prices, and key actions.
+- Charcoal gray (#2C2C2C) for body copy and explanatory text, keeping it clear without feeling harsh.
+- Pale gold (#C9A84C) only as a subtle accent, for tags, thin lines, price emphasis, or decorative gold lines.
+- Dark areas can use light bamboo green (#1E3A0F) with warm white text to create calm brand sections.
+# Font
+- Use "SourceHanSerifCN" for brand titles, page titles, and key numerals. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-SemiBold.woff2)
+- Use "SourceHanSerifCN" for body text, navigation, buttons, and explanatory copy. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+# Animation
+- Use a subtle 160ms press feedback on button tap, keeping it restrained, quick, and natural.
+- For cards, products, and image-text sections, use a "fade in + slide up" entrance animation, with staggered delays to create a quiet sense of ritual.
+- On hover or touch, cards rise slightly by 2px, with softly enhanced borders or shadows, avoiding exaggerated motion.
+- Respect `prefers-reduced-motion` by disabling transitions and entrance animations when motion is reduced.
+# Layout
+- The page should scroll vertically, with ample whitespace and clear section breaks.
+- Use an asymmetrical relationship between content and imagery, echoing a 60% information and 40% visual balance.
+- Spacing follows a 4px grid, with generous breathing room between paragraphs, compact heading line height, and loose body line height.
+- Product cards, brand intro sections, and cart areas should be grouped softly to avoid dense stacking.
+# Elements
+- Buttons use 8px corner radius, cards use 12px-16px corner radius, avoiding an overly cute fully rounded look.
+- Tags use a pale gold background and small rounded corners to present lightweight information such as "Best Seller" and "New".
+- Borders use semi-transparent deep bamboo green or charcoal gray, and cards have no heavy default shadow, keeping the look flat and quiet.
+- Dividers can use a bamboo-stem gradient line or a 1px pale gold line as a refined Eastern detail.
+- Choose low-saturation plant photography, emphasizing natural textures, soil, leaves, and light and shadow, without cluttered backgrounds.</t>
+        </is>
+      </c>
+      <c r="Z120" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>Cel Animation</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>Thick black outlines, flat color blocks, high-saturation palettes, and hard-edged shadows evoke the visual feel of traditional cel animation and cartoon game menus.</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W121" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t># Theme Name: Cel Animation
+# Vibe &amp; Description:
+Thick black outlines, flat color blocks, high-saturation palettes, and hard-edged shadows evoke the visual feel of traditional cel animation and cartoon game menus.
+# Color
+- Use a high-saturation, high-contrast pure color system; gradients, soft gray tones, and low-saturation palettes are prohibited.
+- Backgrounds and borders use deep ink (#1A1A2E) to create clear outlines, while light areas use warm white (#FAFAF5). Accent colors include animation-inspired red (#E63946), blue (#4EA8DE), green (#2ECC71), and yellow (#F1C40F). The overall palette should feel like hand-drawn animation with layered coloring: bright, direct, and game-like.
+# Font
+- Titles use YouSheBiaoTiHei, a heavy, compact, eye-catching display font that emphasizes uppercase, font-black, and strong visual impact. (https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf)
+- Body text uses AlibabaPuHuiTi 3.0. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'YouSheBiaoTiHei-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the fontFamily property in `tailwind.config.js` to extend the fonts
+```js
+{
+  fontFamily: {
+   'youshe-title': ['YouSheBiaoTiHei-Regular', 'sans-serif'],
+    'alibaba-puhuiti-body': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-youshe-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-alibaba-puhuiti-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Interactions should be short and direct, with durations kept between 75-150ms, simulating limited animation frames rather than silky transitions.
+- On tap, use slight displacement, hard-shadow compression, and Squash &amp; Stretch feedback, such as `scale-x-110 scale-y-90`, making buttons feel like cartoon props being pressed.
+# Layout
+- Pages use right-angle cuts, thick black dividers, and clear alignment, with every element resembling an independent color block in an animation storyboard.
+- Cards, buttons, and information areas maintain stable dimensions; mobile touch targets should be no smaller than 44px. The overall layout may be slightly asymmetrical but must preserve a clear hierarchy.
+# Elements
+- Buttons and cards consistently use `border-[3px] border-[#1a1a2e] rounded-none` to create strong cel-style outlines.
+- Shadows use hard offsets with no blur, such as `shadow-[3px_3px_0_#1a1a2e]`; soft drop shadows are prohibited.
+- Element fills use solid color blocks with no gradients; red, blue, green, and yellow may serve as primary action and status colors.</t>
+        </is>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>Cel Animation</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>Thick black outlines, flat color blocks, high-saturation palettes, and hard-edged shadows evoke the visual feel of traditional cel animation and cartoon game menus.</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W122" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t># Theme Name: Cel Animation
+# Vibe &amp; Description:
+Thick black outlines, flat color blocks, high-saturation palettes, and hard-edged shadows evoke the visual feel of traditional cel animation and cartoon game menus.
+# Color
+- Use a high-saturation, high-contrast pure color system; gradients, soft gray tones, and low-saturation palettes are prohibited.
+- Backgrounds and borders use deep ink (#1A1A2E) to create clear outlines, while light areas use warm white (#FAFAF5). Accent colors include animation-inspired red (#E63946), blue (#4EA8DE), green (#2ECC71), and yellow (#F1C40F). The overall palette should feel like hand-drawn animation with layered coloring: bright, direct, and game-like.
+# Font
+- Titles use YouSheBiaoTiHei, a heavy, compact, eye-catching display font that emphasizes uppercase, font-black, and strong visual impact. (https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf)
+- Body text uses AlibabaPuHuiTi 3.0. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- Interactions should be short and direct, with durations kept between 75-150ms, simulating limited animation frames rather than silky transitions.
+- On tap, use slight displacement, hard-shadow compression, and Squash &amp; Stretch feedback, such as `scale-x-110 scale-y-90`, making buttons feel like cartoon props being pressed.
+# Layout
+- Pages use right-angle cuts, thick black dividers, and clear alignment, with every element resembling an independent color block in an animation storyboard.
+- Cards, buttons, and information areas maintain stable dimensions; mobile touch targets should be no smaller than 44px. The overall layout may be slightly asymmetrical but must preserve a clear hierarchy.
+# Elements
+- Buttons and cards consistently use `border-[3px] border-[#1a1a2e] rounded-none` to create strong cel-style outlines.
+- Shadows use hard offsets with no blur, such as `shadow-[3px_3px_0_#1a1a2e]`; soft drop shadows are prohibited.
+- Element fills use solid color blocks with no gradients; red, blue, green, and yellow may serve as primary action and status colors.</t>
+        </is>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>Cathedral Gothic</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>Medieval cathedral aesthetics, with deep purple, blood red, and black setting the tone, paired with gold lines, pointed arches, and rose windows for a dark, solemn, mysterious classical mood.</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W123" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y123" t="inlineStr">
+        <is>
+          <t># Theme Name: Cathedral Gothic
+# Vibe &amp; Description:
+Medieval cathedral aesthetics, with deep purple, blood red, and black setting the tone, paired with gold lines, pointed arches, and rose windows for a dark, solemn, mysterious classical mood.
+# Color
+- Use deep purple, blood red, black, and gold exclusively; avoid pure white, light gray, pink, green, blue, and neon colors.
+- Make black (#000000) or deep purple (#2D1B4E) the main background, with blood red (#8B0000) used in spots to create a heavy, religious mural-like feel. Use gold (#FFD700 / #c9a227) for text and decoration, and semi-transparent gold for borders (border-[#c9a227]/40), presenting the solemn visual of a "dark cathedral".
+# Font
+- Use “SourceHanSerifCN-Bold” as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use “AlibabaPuHuiTi-Regular” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'SourceHanSerifCN-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add `fontFamily` property extensions in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'title-serif-bold': ['SourceHanSerifCN-Bold', 'serif'],
+    'body-alibaba': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-serif-bold text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch, do not use a lively bounce; use a gold halo and deeper shadow as feedback, keeping it solemn and restrained. On tap, allow a slight scale to `active:scale-95`.
+- When elements appear, use a slow fade-in or dark-area emergence effect, like candlelight illuminating carved stone patterns. Use `transition-all duration-300 ease-in-out` uniformly for transitions.
+# Layout
+- The page should be vertically oriented, symmetrical, and ritualistic, simulating a cathedral central axis. On mobile, keep a single-column layout, leaving ample breathing room between cards and sections.
+- Section edges may incorporate pointed arches, thin gold lines, or manuscript-style borders. Use sharp-cornered cards and avoid rounded contours; establish hierarchy through dark-light variation, gold outlines, and font-size differences.
+# Elements
+- Buttons use transparent backgrounds, gold outlines, and serif text; on hover or press, a semi-transparent gold background and dark text appear.
+- Cards use `bg-[#0a0a0a]/90`, `border-2 border-[#c9a227]/40`, `rounded-none`, with shadows rendered as deep dark diffusion or gold halos.
+- Prefer pointed arches, rose windows, flying buttress lines, and manuscript borders for decorative elements to strengthen the medieval Gothic atmosphere.
+- Divider lines, icons, and navigation should emphasize thin gold lines, avoiding modern rounded corners, soft cartoon forms, and highly saturated bright colors.</t>
+        </is>
+      </c>
+      <c r="Z123" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>Cathedral Gothic</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>Medieval cathedral aesthetics, with deep purple, blood red, and black setting the tone, paired with gold lines, pointed arches, and rose windows for a dark, solemn, mysterious classical mood.</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W124" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t># Theme Name: Cathedral Gothic
+# Vibe &amp; Description:
+Medieval cathedral aesthetics, with deep purple, blood red, and black setting the tone, paired with gold lines, pointed arches, and rose windows for a dark, solemn, mysterious classical mood.
+# Color
+- Use deep purple, blood red, black, and gold exclusively; avoid pure white, light gray, pink, green, blue, and neon colors.
+- Make black (#000000) or deep purple (#2D1B4E) the main background, with blood red (#8B0000) used in spots to create a heavy, religious mural-like feel. Use gold (#FFD700 / #c9a227) for text and decoration, and semi-transparent gold for borders (border-[#c9a227]/40), presenting the solemn visual of a "dark cathedral".
+# Font
+- Use “SourceHanSerifCN-Bold” as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use “AlibabaPuHuiTi-Regular” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- On touch, do not use a lively bounce; use a gold halo and deeper shadow as feedback, keeping it solemn and restrained. On tap, allow a slight scale to `active:scale-95`.
+- When elements appear, use a slow fade-in or dark-area emergence effect, like candlelight illuminating carved stone patterns. Use `transition-all duration-300 ease-in-out` uniformly for transitions.
+# Layout
+- The page should be vertically oriented, symmetrical, and ritualistic, simulating a cathedral central axis. On mobile, keep a single-column layout, leaving ample breathing room between cards and sections.
+- Section edges may incorporate pointed arches, thin gold lines, or manuscript-style borders. Use sharp-cornered cards and avoid rounded contours; establish hierarchy through dark-light variation, gold outlines, and font-size differences.
+# Elements
+- Buttons use transparent backgrounds, gold outlines, and serif text; on hover or press, a semi-transparent gold background and dark text appear.
+- Cards use `bg-[#0a0a0a]/90`, `border-2 border-[#c9a227]/40`, `rounded-none`, with shadows rendered as deep dark diffusion or gold halos.
+- Prefer pointed arches, rose windows, flying buttress lines, and manuscript borders for decorative elements to strengthen the medieval Gothic atmosphere.
+- Divider lines, icons, and navigation should emphasize thin gold lines, avoiding modern rounded corners, soft cartoon forms, and highly saturated bright colors.</t>
+        </is>
+      </c>
+      <c r="Z124" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Op Art</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>Optical illusion, stark black-and-white contrast, precise geometric patterns, emphasizing visual tension and a sense of planar motion, using restrained vibrating colors to create strong memorability.</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W125" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y125" t="inlineStr">
+        <is>
+          <t># Theme Name: Op Art
+# Vibe &amp; Description:
+Optical illusion, stark black-and-white contrast, precise geometric patterns, emphasizing visual tension and a sense of planar motion, using restrained vibrating colors to create strong memorability.
+# Color
+- Use pure black and pure white as absolute primary colors, maintaining a clear, sharp visual confrontation with no grayscale transitions.
+- Background and text use high-contrast pairings: white text on black or black text on white. Accent colors are limited to vibrating color pairs, such as vermilion (#FF3300), bright blue (#0066FF), vivid yellow (#FFCC00), and olive green (#5E6D00). Soft gradients, translucency, blur, and low-contrast shadows are prohibited.
+# Font
+- Use “AlibabaPuHuiTi” as the title font to maintain an uppercase feel, geometric character, and strong rhythm. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_SemiBold.ttf)
+- Use “AlibabaPuHuiTi” as the body font to ensure clear reading on mobile. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'AlibabaPuHuiTi-SemiBold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_SemiBold.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the fontFamily property in `tailwind.config.js` to unify font semantics
+```js
+{
+  fontFamily: {
+    'alibaba-puhuiti-title': ['AlibabaPuHuiTi-SemiBold', 'sans-serif'],
+    'alibaba-puhuiti-body': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-alibaba-puhuiti-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-alibaba-puhuiti-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On tap, use a firm press feedback, such as a slight displacement `translate-x-[2px] translate-y-[2px]`, avoiding soft elastic animation.
+- Interaction states focus on black-and-white inversion, border emphasis, or hard-edge shadow changes. Transitions use only brief color changes, maintaining a mechanical, precise rhythm.
+# Layout
+- Pages are primarily mobile single-column layouts, with clear information hierarchy, large titles, ample spacing, and restrained decoration.
+- Cards, buttons, and sections keep right-angled borders, using `border-2 border-black rounded-none`, optionally paired with a `4px` hard-edge offset shadow to form a poster-like geometric order.
+# Elements
+- Use concentric circles, checkerboards, stripes, and moiré patterns as local decoration; do not cover large areas, to avoid visual fatigue.
+- Buttons use black-and-white inversion styles, with vermilion or bright blue used when needed for borders, corner labels, or small accent blocks.
+- Cards use pure white or pure black backgrounds, paired with clear borders and no-radius structures to maintain a strong flat feel.
+- All visual elements avoid soft shadows, rounded corners, gradients, and glassmorphism, presenting an overall sharp, precise, optical mobile interface.</t>
+        </is>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>Op Art</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>Optical illusion, stark black-and-white contrast, precise geometric patterns, emphasizing visual tension and a sense of planar motion, using restrained vibrating colors to create strong memorability.</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W126" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y126" t="inlineStr">
+        <is>
+          <t># Theme Name: Op Art
+# Vibe &amp; Description:
+Optical illusion, stark black-and-white contrast, precise geometric patterns, emphasizing visual tension and a sense of planar motion, using restrained vibrating colors to create strong memorability.
+# Color
+- Use pure black and pure white as absolute primary colors, maintaining a clear, sharp visual confrontation with no grayscale transitions.
+- Background and text use high-contrast pairings: white text on black or black text on white. Accent colors are limited to vibrating color pairs, such as vermilion (#FF3300), bright blue (#0066FF), vivid yellow (#FFCC00), and olive green (#5E6D00). Soft gradients, translucency, blur, and low-contrast shadows are prohibited.
+# Font
+- Use “AlibabaPuHuiTi” as the title font to maintain an uppercase feel, geometric character, and strong rhythm. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_SemiBold.ttf)
+- Use “AlibabaPuHuiTi” as the body font to ensure clear reading on mobile. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- On tap, use a firm press feedback, such as a slight displacement `translate-x-[2px] translate-y-[2px]`, avoiding soft elastic animation.
+- Interaction states focus on black-and-white inversion, border emphasis, or hard-edge shadow changes. Transitions use only brief color changes, maintaining a mechanical, precise rhythm.
+# Layout
+- Pages are primarily mobile single-column layouts, with clear information hierarchy, large titles, ample spacing, and restrained decoration.
+- Cards, buttons, and sections keep right-angled borders, using `border-2 border-black rounded-none`, optionally paired with a `4px` hard-edge offset shadow to form a poster-like geometric order.
+# Elements
+- Use concentric circles, checkerboards, stripes, and moiré patterns as local decoration; do not cover large areas, to avoid visual fatigue.
+- Buttons use black-and-white inversion styles, with vermilion or bright blue used when needed for borders, corner labels, or small accent blocks.
+- Cards use pure white or pure black backgrounds, paired with clear borders and no-radius structures to maintain a strong flat feel.
+- All visual elements avoid soft shadows, rounded corners, gradients, and glassmorphism, presenting an overall sharp, precise, optical mobile interface.</t>
+        </is>
+      </c>
+      <c r="Z126" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>Hand-Drawn Draft</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>Irregular lines, paper texture, and a doodle-and-sticky-note feel, emphasizing an authentic, relaxed, human hand-drawn draft quality.</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W127" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t># Theme Name: Hand-Drawn Draft
+# Vibe &amp; Description:
+Irregular lines, paper texture, and a doodle-and-sticky-note feel, emphasizing an authentic, relaxed, human hand-drawn draft quality.
+# Color
+- Keep the palette restrained, using only warm paper white, pencil black, aged paper gray, correction red, and ballpoint blue.
+- Use warm paper color (#FDFBF7) for the background and soft pencil black (#2D2D2D) for text, avoiding the mechanical feel of pure black. Use aged paper color (#E5E0D8) as the supporting gray, correction red (#FF4D4D) as the accent color, and a small amount of blue (#2D5DA1) for handwritten marks or focused states.
+# Font
+- Use “MuyaoSoftbrush” as the title font, with a relatively bold weight, like headings written with a thick felt-tip pen. (https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf)
+- Use “ResourceHanRoundedCN” as the body font to stay clear and readable while preserving a handwritten feel. (https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'MuyaoSoftbrush-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf' },
+  'ResourceHanRoundedCN-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Regular.ttf' },
+});
+```
+Add the fontFamily extension in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+   'title-muyao': ['MuyaoSoftbrush-Regular', 'sans-serif'],
+   'body-resource-rounded': ['ResourceHanRoundedCN-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-muyao text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-resource-rounded text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch, elements shift slightly, and the shadow shortens from `4px 4px 0` to `2px 2px 0`, creating feedback like a piece of paper being pressed down.
+- Cards or buttons may rotate slightly by 1-2 degrees on hover, with a quick, direct motion like a hand-drawn sticker being gently flicked.
+# Layout
+- The page resembles a collage layout on a sketchbook, allowing slight misalignment, overlap, and asymmetry without pursuing a precise grid.
+- Cards, images, and hint labels may have small-angle rotations, with generous whitespace, maintaining an easy order that feels “casually tidied up.”
+# Elements
+- All buttons, cards, and input fields use irregular rounded corners, avoiding standard radii, with borders that feel hand-drawn and slightly shaky.
+- Borders use relatively thick pencil-black solid lines; secondary dividers may use dashed lines, and shadows use a hard offset with no blur.
+- Overlay a subtle paper dot texture on the background, such as `radial-gradient(#E5E0D8 1px, transparent 1px)`.
+- Tape, pushpins, dashed arrows, sticky-note labels, and doodle underlines may be used as decoration, but only as light accents.</t>
+        </is>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>Hand-Drawn Draft</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Irregular lines, paper texture, and a doodle-and-sticky-note feel, emphasizing an authentic, relaxed, human hand-drawn draft quality.</t>
+        </is>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W128" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y128" t="inlineStr">
+        <is>
+          <t># Theme Name: Hand-Drawn Draft
+# Vibe &amp; Description:
+Irregular lines, paper texture, and a doodle-and-sticky-note feel, emphasizing an authentic, relaxed, human hand-drawn draft quality.
+# Color
+- Keep the palette restrained, using only warm paper white, pencil black, aged paper gray, correction red, and ballpoint blue.
+- Use warm paper color (#FDFBF7) for the background and soft pencil black (#2D2D2D) for text, avoiding the mechanical feel of pure black. Use aged paper color (#E5E0D8) as the supporting gray, correction red (#FF4D4D) as the accent color, and a small amount of blue (#2D5DA1) for handwritten marks or focused states.
+# Font
+- Use “MuyaoSoftbrush” as the title font, with a relatively bold weight, like headings written with a thick felt-tip pen. (https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf)
+- Use “ResourceHanRoundedCN” as the body font to stay clear and readable while preserving a handwritten feel. (https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Regular.ttf)
+# Animation
+- On touch, elements shift slightly, and the shadow shortens from `4px 4px 0` to `2px 2px 0`, creating feedback like a piece of paper being pressed down.
+- Cards or buttons may rotate slightly by 1-2 degrees on hover, with a quick, direct motion like a hand-drawn sticker being gently flicked.
+# Layout
+- The page resembles a collage layout on a sketchbook, allowing slight misalignment, overlap, and asymmetry without pursuing a precise grid.
+- Cards, images, and hint labels may have small-angle rotations, with generous whitespace, maintaining an easy order that feels “casually tidied up.”
+# Elements
+- All buttons, cards, and input fields use irregular rounded corners, avoiding standard radii, with borders that feel hand-drawn and slightly shaky.
+- Borders use relatively thick pencil-black solid lines; secondary dividers may use dashed lines, and shadows use a hard offset with no blur.
+- Overlay a subtle paper dot texture on the background, such as `radial-gradient(#E5E0D8 1px, transparent 1px)`.
+- Tape, pushpins, dashed arrows, sticky-note labels, and doodle underlines may be used as decoration, but only as light accents.</t>
+        </is>
+      </c>
+      <c r="Z128" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>Kawaii Minimal</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>Pastel palette, rounded shapes, airy whitespace, and a minimalist style with a Japanese kawaii spirit. Overall gentle, fresh, and approachable, emphasizing cuteness without clutter.</t>
+        </is>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W129" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t># Theme Name: Kawaii Minimal
+# Vibe &amp; Description:
+Pastel palette, rounded shapes, airy whitespace, and a minimalist style with a Japanese kawaii spirit. Overall gentle, fresh, and approachable, emphasizing cuteness without clutter.
+# Color
+- Use low-saturation pastel colors, avoiding dark backgrounds, fluorescent colors, and neon glow.
+- Use warm white (#FFF7ED) or an extremely light orange-white for the background, soft pink (#F9A8D4) as the primary color, and pale purple (#A78BFA), light cyan (#67E8F9), and pale yellow (#FDE68A) as accents. Use soft dark gray for text to keep it clear without feeling harsh.
+# Font
+- Use “ResourceHanRoundedCN-Bold” as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Bold.ttf)
+- Use “HarmonyOS Sans” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+## Font Import Method
+Load fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'ResourceHanRoundedCN-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Bold.ttf' },
+  'HarmonyOSSans-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf' },
+});
+```
+Add the fontFamily extension in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'title-resource-rounded': ['ResourceHanRoundedCN-Bold', 'sans-serif'],
+    'body-harmony': ['HarmonyOSSans-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-resource-rounded text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-harmony text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Use a subtle bounce-back feedback on tap, with elements shrinking first and then returning, like soft candy being pressed.
+- For hover or touch feedback, use `scale-105` and `active:scale-95`, with a transition duration of about 200ms and an easing curve with a bouncy feel.
+- When elements appear, use fade-in, slight upward float, or small swaying motions, avoiding stiff linear animations.
+# Layout
+- Keep generous whitespace and low information density, like soft pastel cards gently placed on a warm white background.
+- Use large rounded corners consistently for cards, buttons, and input fields, commonly `rounded-2xl`, `rounded-3xl`, and `rounded-full`.
+- On mobile, touch targets should be no smaller than 44px, with comfortable spacing; establish hierarchy through color depth, font size, and whitespace.
+# Elements
+- Buttons use solid pastel colors or soft gradients, capsule-shaped rounded corners, and slight scale feedback.
+- Cards use white or warm white backgrounds with soft shadows `shadow-sm` / `shadow-md`, and may add a light pink border `border-2 border-pink-200`.
+- Input fields use rounded borders and pastel focus rings, such as `focus:ring-4 focus:ring-pink-100`.
+- Avoid thick black borders, strong shadows, small corner radii, and any neon glow effects.</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>Kawaii Minimal</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>Pastel palette, rounded shapes, airy whitespace, and a minimalist style with a Japanese kawaii spirit. Overall gentle, fresh, and approachable, emphasizing cuteness without clutter.</t>
+        </is>
+      </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W130" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y130" t="inlineStr">
+        <is>
+          <t># Theme Name: Kawaii Minimal
+# Vibe &amp; Description:
+Pastel palette, rounded shapes, airy whitespace, and a minimalist style with a Japanese kawaii spirit. Overall gentle, fresh, and approachable, emphasizing cuteness without clutter.
+# Color
+- Use low-saturation pastel colors, avoiding dark backgrounds, fluorescent colors, and neon glow.
+- Use warm white (#FFF7ED) or an extremely light orange-white for the background, soft pink (#F9A8D4) as the primary color, and pale purple (#A78BFA), light cyan (#67E8F9), and pale yellow (#FDE68A) as accents. Use soft dark gray for text to keep it clear without feeling harsh.
+# Font
+- Use “ResourceHanRoundedCN-Bold” as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Bold.ttf)
+- Use “HarmonyOS Sans” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+# Animation
+- Use a subtle bounce-back feedback on tap, with elements shrinking first and then returning, like soft candy being pressed.
+- For hover or touch feedback, use `scale-105` and `active:scale-95`, with a transition duration of about 200ms and an easing curve with a bouncy feel.
+- When elements appear, use fade-in, slight upward float, or small swaying motions, avoiding stiff linear animations.
+# Layout
+- Keep generous whitespace and low information density, like soft pastel cards gently placed on a warm white background.
+- Use large rounded corners consistently for cards, buttons, and input fields, commonly `rounded-2xl`, `rounded-3xl`, and `rounded-full`.
+- On mobile, touch targets should be no smaller than 44px, with comfortable spacing; establish hierarchy through color depth, font size, and whitespace.
+# Elements
+- Buttons use solid pastel colors or soft gradients, capsule-shaped rounded corners, and slight scale feedback.
+- Cards use white or warm white backgrounds with soft shadows `shadow-sm` / `shadow-md`, and may add a light pink border `border-2 border-pink-200`.
+- Input fields use rounded borders and pastel focus rings, such as `focus:ring-4 focus:ring-pink-100`.
+- Avoid thick black borders, strong shadows, small corner radii, and any neon glow effects.</t>
+        </is>
+      </c>
+      <c r="Z130" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>Ancient Elegance</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>Song-era Eastern aesthetics, with xuan paper textures intertwined with subtle blue-green landscape motifs, warm and refined, with a strong antique album feel, emphasizing whitespace, colophons, seals, and the spirit of brush and ink.</t>
+        </is>
+      </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W131" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y131" t="inlineStr">
+        <is>
+          <t># Theme Name: Ancient Elegance
+# Vibe &amp; Description:
+Song-era Eastern aesthetics, with xuan paper textures intertwined with subtle blue-green landscape motifs, warm and refined, with a strong antique album feel, emphasizing whitespace, colophons, seals, and the spirit of brush and ink.
+# Color
+- Use low-saturation, warm traditional colors; avoid pure white, pure black, and highly saturated neon tones.
+- Use a light beige xuan paper background (#F9F6EF / #F5EEDC), layered with low-opacity antique painting motifs. Use ink black (#2C2C2C) for text, stone blue (#2D5A6E) and stone green (#5B7A5A) for primary visuals, ancient brown (#8B6B4D) for borders and dividers, and cinnabar red (#C43B2B) for emphasis.
+# Font
+- Use "SourceHanSerifCN" as the heading font, conveying the antique charm of brush calligraphy. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-SemiBold.woff2)
+- Use "SourceHanSerifCN" as the body font, preserving the warm feel of Song-style type and mobile readability. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'SourceHanSerifCN-SemiBold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-SemiBold.woff2' },
+  'SourceHanSerifCN-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2' },
+});
+```
+Extend the fontFamily property in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'title-serif-semibold': ['SourceHanSerifCN-SemiBold', 'serif'],
+    'body-serif': ['SourceHanSerifCN-Regular', 'serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-serif-semibold text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-serif text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- When touching cards or icons, elements lift slightly, borders deepen, and cinnabar red is used for highlight feedback.
+- When clicking seals or key buttons, use a brief "stamp" animation (scale 0.95→1.05→1) to create the ritual feel of red seal ink on paper.
+- When page elements appear, use a "scroll unrolling" or "fade in + slight shift" motion; hovering states can include a low-opacity ink wash transition.
+# Layout
+- On mobile, use a vertically stacked antique album layout with stacked cards, preserving ample whitespace and symmetry.
+- Banners can use centered or colophon-style offset layouts, with prominent titles and enough breathing room like xuan paper.
+- Content cards follow a classical colophon structure: title, body, author info, and cinnabar seal appear in sequence, with generous line height and a relaxed reading rhythm.
+# Elements
+- Use a light beige xuan paper texture for the background, overlaid with low-saturation blue-green landscapes, antique paintings, or subtle ink-cloud motifs.
+- Cards use an aged paper texture, fine brown line borders, and corner radii controlled at 0-4px to avoid an overly modern feel.
+- Functional entry points use circular traditional line-art icons, which may include landscapes, pavilions, scrolls, brush pens, and auspicious clouds.
+- Decorative elements should center on cinnabar seals, ink-wash patterns, scroll edges, and delicate traditional lines; keep them restrained, and avoid glassmorphism, flashy gradients, or heavy shadows.</t>
+        </is>
+      </c>
+      <c r="Z131" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>Ancient Elegance</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>Song-era Eastern aesthetics, with xuan paper textures intertwined with subtle blue-green landscape motifs, warm and refined, with a strong antique album feel, emphasizing whitespace, colophons, seals, and the spirit of brush and ink.</t>
+        </is>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W132" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y132" t="inlineStr">
+        <is>
+          <t># Theme Name: Ancient Elegance
+# Vibe &amp; Description:
+Song-era Eastern aesthetics, with xuan paper textures intertwined with subtle blue-green landscape motifs, warm and refined, with a strong antique album feel, emphasizing whitespace, colophons, seals, and the spirit of brush and ink.
+# Color
+- Use low-saturation, warm traditional colors; avoid pure white, pure black, and highly saturated neon tones.
+- Use a light beige xuan paper background (#F9F6EF / #F5EEDC), layered with low-opacity antique painting motifs. Use ink black (#2C2C2C) for text, stone blue (#2D5A6E) and stone green (#5B7A5A) for primary visuals, ancient brown (#8B6B4D) for borders and dividers, and cinnabar red (#C43B2B) for emphasis.
+# Font
+- Use "SourceHanSerifCN" as the heading font, conveying the antique charm of brush calligraphy. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-SemiBold.woff2)
+- Use "SourceHanSerifCN" as the body font, preserving the warm feel of Song-style type and mobile readability. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+# Animation
+- When touching cards or icons, elements lift slightly, borders deepen, and cinnabar red is used for highlight feedback.
+- When clicking seals or key buttons, use a brief "stamp" animation (scale 0.95→1.05→1) to create the ritual feel of red seal ink on paper.
+- When page elements appear, use a "scroll unrolling" or "fade in + slight shift" motion; hovering states can include a low-opacity ink wash transition.
+# Layout
+- On mobile, use a vertically stacked antique album layout with stacked cards, preserving ample whitespace and symmetry.
+- Banners can use centered or colophon-style offset layouts, with prominent titles and enough breathing room like xuan paper.
+- Content cards follow a classical colophon structure: title, body, author info, and cinnabar seal appear in sequence, with generous line height and a relaxed reading rhythm.
+# Elements
+- Use a light beige xuan paper texture for the background, overlaid with low-saturation blue-green landscapes, antique paintings, or subtle ink-cloud motifs.
+- Cards use an aged paper texture, fine brown line borders, and corner radii controlled at 0-4px to avoid an overly modern feel.
+- Functional entry points use circular traditional line-art icons, which may include landscapes, pavilions, scrolls, brush pens, and auspicious clouds.
+- Decorative elements should center on cinnabar seals, ink-wash patterns, scroll edges, and delicate traditional lines; keep them restrained, and avoid glassmorphism, flashy gradients, or heavy shadows.</t>
+        </is>
+      </c>
+      <c r="Z132" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>African Weave</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>A visual style inspired by West African Kente weaving and Adire tie-dye, with bold geometry, warm earth tones, and coarse textile textures, conveying the cultural depth and vivid rhythm of handcrafted fabric.</t>
+        </is>
+      </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W133" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y133" t="inlineStr">
+        <is>
+          <t># Theme Name: African Weave
+# Vibe &amp; Description:
+A visual style inspired by West African Kente weaving and Adire tie-dye, with bold geometry, warm earth tones, and coarse textile textures, conveying the cultural depth and vivid rhythm of handcrafted fabric.
+# Color
+- Use deep wood, terracotta orange, sand gold, sand, and forest green; avoid pure white, pastels, and neon colors.
+- Use deep wood (#2C1810) as a weighty foundation for the background, sand (#E8D5B5) for cards, Kente orange (#C4501F) and gold (#F0C75E) as accent colors, and forest green (#1A5632) for decorative text or local highlights, creating a collision between earth tones and vivid color blocks.
+# Font
+- Use “SourceHanSerifCN-Bold” as the title font, paired with an uppercase feel, heavy weight, and wide letter spacing. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use “HarmonyOS Sans” as the body font to maintain a clear, stable reading experience with a humanistic warmth. (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'SourceHanSerifCN-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2' },
+  'HarmonyOSSans-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf' },
+});
+```
+Add a fontFamily extension to `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'serif-title': ['SourceHanSerifCN-Bold', 'serif', 'sans-serif'],
+    'harmony-body': ['HarmonyOSSans-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-serif-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-harmony-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Use hard-edged shadow changes as the primary feedback on click, avoiding a soft floating feel; buttons and cards can shift from a `2px` shadow to a `4px/6px` shadow.
+- When elements appear, use a brisk fade-in with slight scaling to simulate textile patterns unfolding; keep the interaction rhythm crisp and weighty.
+# Layout
+- The page uses strong geometric zoning: a dark background carries the main visual, sand-colored cards carry content, and thick borders clearly divide information hierarchy.
+- On mobile, use mainly single-column cards with ample spacing between sections; titles are large, bold, and widely spaced, forming a rhythm reminiscent of Kente stripes.
+# Elements
+- Cards and buttons use `border-2`, `rounded-lg`, and hard-edged offset shadows; avoid fully rounded corners, glassmorphism, and blur effects.
+- Decorative elements use geometric stripes, color-block stitching, woven grids, or tie-dye textures; control their proportion to avoid overpowering the content.
+- The background may layer in rough textile noise; dividers and borders should remain thick and clear, presenting the imperfect edges of handmade cloth.</t>
+        </is>
+      </c>
+      <c r="Z133" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>African Weave</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>A visual style inspired by West African Kente weaving and Adire tie-dye, with bold geometry, warm earth tones, and coarse textile textures, conveying the cultural depth and vivid rhythm of handcrafted fabric.</t>
+        </is>
+      </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W134" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y134" t="inlineStr">
+        <is>
+          <t># Theme Name: African Weave
+# Vibe &amp; Description:
+A visual style inspired by West African Kente weaving and Adire tie-dye, with bold geometry, warm earth tones, and coarse textile textures, conveying the cultural depth and vivid rhythm of handcrafted fabric.
+# Color
+- Use deep wood, terracotta orange, sand gold, sand, and forest green; avoid pure white, pastels, and neon colors.
+- Use deep wood (#2C1810) as a weighty foundation for the background, sand (#E8D5B5) for cards, Kente orange (#C4501F) and gold (#F0C75E) as accent colors, and forest green (#1A5632) for decorative text or local highlights, creating a collision between earth tones and vivid color blocks.
+# Font
+- Use “SourceHanSerifCN-Bold” as the title font, paired with an uppercase feel, heavy weight, and wide letter spacing. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use “HarmonyOS Sans” as the body font to maintain a clear, stable reading experience with a humanistic warmth. (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+# Animation
+- Use hard-edged shadow changes as the primary feedback on click, avoiding a soft floating feel; buttons and cards can shift from a `2px` shadow to a `4px/6px` shadow.
+- When elements appear, use a brisk fade-in with slight scaling to simulate textile patterns unfolding; keep the interaction rhythm crisp and weighty.
+# Layout
+- The page uses strong geometric zoning: a dark background carries the main visual, sand-colored cards carry content, and thick borders clearly divide information hierarchy.
+- On mobile, use mainly single-column cards with ample spacing between sections; titles are large, bold, and widely spaced, forming a rhythm reminiscent of Kente stripes.
+# Elements
+- Cards and buttons use `border-2`, `rounded-lg`, and hard-edged offset shadows; avoid fully rounded corners, glassmorphism, and blur effects.
+- Decorative elements use geometric stripes, color-block stitching, woven grids, or tie-dye textures; control their proportion to avoid overpowering the content.
+- The background may layer in rough textile noise; dividers and borders should remain thick and clear, presenting the imperfect edges of handmade cloth.</t>
+        </is>
+      </c>
+      <c r="Z134" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>Newspaper Aesthetic</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>Newsprint texture, high-contrast black and white, zero-radius geometric structure, emphasizing clear grids, editorial authority, and the solemn order of a newspaper front page.</t>
+        </is>
+      </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W135" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y135" t="inlineStr">
+        <is>
+          <t># Theme Name: Newspaper Aesthetic
+# Vibe &amp; Description:
+Newsprint texture, high-contrast black and white, zero-radius geometric structure, emphasizing clear grids, editorial authority, and the solemn order of a newspaper front page.
+# Color
+- Build a strict color system from newsprint off-white, ink black, and editorial red, avoiding rich gradients and decorative colors.
+- Use warm paper color (#F9F9F7) for backgrounds, ink black (#111111) for text and borders, and light gray (#E5E5E0) for secondary dividers. Use editorial red (#CC0000) only for breaking-news labels, key buttons, or minimal status cues, keeping the whole look restrained, credible, and sharp.
+# Font
+- Use “AlibabaPuHuiTi” as the title font to create a striking newspaper front-page headline feel. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_SemiBold.ttf)
+- Use “AlibabaPuHuiTi” as the body font to ensure clear mobile reading. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'AlibabaPuHuiTi-SemiBold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_SemiBold.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the `fontFamily` extension in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'alibaba-puhuiti-title': ['AlibabaPuHuiTi-SemiBold', 'sans-serif'],
+    'alibaba-puhuiti-body': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-alibaba-puhuiti-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-alibaba-puhuiti-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Interaction feedback should be fast, firm, and direct. Use black-white inversion on button taps; cards should shift slightly with a hard shadow offset when pressed, simulating the tactile feel of a newspaper clipping being pushed down.
+- Avoid soft elastic animation, blur, gradients, and floating shadows. Page transitions and element entrances may use brief fades or vertical shifts, maintaining the calm rhythm of an editorial layout.
+# Layout
+- On mobile, use a compact newspaper-column layout, forming a clear page structure through distinct border weights, dividers, and modular assembly.
+- Keep a masthead, date, volume number, or edition information at the top. The content area may use asymmetrical cards, headline zones, scrolling news tickers, and inverted black sections to create front-page information density.
+- All modules should share boundaries and reduce unnecessary whitespace. Headlines may occupy a large visual area, while body text should stay justified or feel neatly columned.
+# Elements
+- All buttons, cards, input fields, and image containers must keep 0 radius; use 1px ink-black borders, with 4px thick lines for key areas.
+- Overlay the background with subtle halftone or paper noise texture; use line grids locally to enhance the newsprint feel.
+- Images use a grayscale filter by default; touch or hover states may add a subtle vintage sepia effect.
+- Labels, navigation, dates, authors, and category information use small uppercase text, wide letter spacing, and a monospaced style.
+- Key links use thick underlines or editorial red accents. Buttons default to white text on a black background, reversing to black text on white when triggered.</t>
+        </is>
+      </c>
+      <c r="Z135" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>Newspaper Aesthetic</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>Newsprint texture, high-contrast black and white, zero-radius geometric structure, emphasizing clear grids, editorial authority, and the solemn order of a newspaper front page.</t>
+        </is>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W136" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y136" t="inlineStr">
+        <is>
+          <t># Theme Name: Newspaper Aesthetic
+# Vibe &amp; Description:
+Newsprint texture, high-contrast black and white, zero-radius geometric structure, emphasizing clear grids, editorial authority, and the solemn order of a newspaper front page.
+# Color
+- Build a strict color system from newsprint off-white, ink black, and editorial red, avoiding rich gradients and decorative colors.
+- Use warm paper color (#F9F9F7) for backgrounds, ink black (#111111) for text and borders, and light gray (#E5E5E0) for secondary dividers. Use editorial red (#CC0000) only for breaking-news labels, key buttons, or minimal status cues, keeping the whole look restrained, credible, and sharp.
+# Font
+- Use “AlibabaPuHuiTi” as the title font to create a striking newspaper front-page headline feel. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_SemiBold.ttf)
+- Use “AlibabaPuHuiTi” as the body font to ensure clear mobile reading. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- Interaction feedback should be fast, firm, and direct. Use black-white inversion on button taps; cards should shift slightly with a hard shadow offset when pressed, simulating the tactile feel of a newspaper clipping being pushed down.
+- Avoid soft elastic animation, blur, gradients, and floating shadows. Page transitions and element entrances may use brief fades or vertical shifts, maintaining the calm rhythm of an editorial layout.
+# Layout
+- On mobile, use a compact newspaper-column layout, forming a clear page structure through distinct border weights, dividers, and modular assembly.
+- Keep a masthead, date, volume number, or edition information at the top. The content area may use asymmetrical cards, headline zones, scrolling news tickers, and inverted black sections to create front-page information density.
+- All modules should share boundaries and reduce unnecessary whitespace. Headlines may occupy a large visual area, while body text should stay justified or feel neatly columned.
+# Elements
+- All buttons, cards, input fields, and image containers must keep 0 radius; use 1px ink-black borders, with 4px thick lines for key areas.
+- Overlay the background with subtle halftone or paper noise texture; use line grids locally to enhance the newsprint feel.
+- Images use a grayscale filter by default; touch or hover states may add a subtle vintage sepia effect.
+- Labels, navigation, dates, authors, and category information use small uppercase text, wide letter spacing, and a monospaced style.
+- Key links use thick underlines or editorial red accents. Buttons default to white text on a black background, reversing to black text on white when triggered.</t>
+        </is>
+      </c>
+      <c r="Z136" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>Airy Kawaii</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>Japanese kawaii meets minimalist whitespace: pastel, rounded, light, and gentle. The overall feel is like a soft breath of oxygen—friendly but not childish, cute but not cluttered.</t>
+        </is>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W137" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y137" t="inlineStr">
+        <is>
+          <t># Theme Name: Airy Kawaii
+# Vibe &amp; Description:
+Japanese kawaii meets minimalist whitespace: pastel, rounded, light, and gentle. The overall feel is like a soft breath of oxygen—friendly but not childish, cute but not cluttered.
+# Color
+- Use low-saturation pastel palettes; avoid dark backgrounds, fluorescent colors, and strong contrasts.
+- Backgrounds are mainly warm white and light cream (#FFF7ED / #FFF9F2). Use soft pink (#F9A8D4) as the primary color, with light purple (#A78BFA), light cyan (#67E8F9), and light yellow (#FDE68A) as accents. Text uses soft dark gray (#4B5563) to reduce the pressure of pure black.
+- Cards mostly use white or light pink backgrounds, with pale pastel borders such as #FBCFE8, creating a light, soft, and clean visual atmosphere.
+# Font
+- Use "ResourceHanRoundedCN-Bold" as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Bold.ttf)
+- Use "HarmonyOS Sans" as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+## Font Import Method
+Load fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'ResourceHanRoundedCN-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Bold.ttf' },
+  'HarmonyOSSans-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf' },
+});
+```
+Add the fontFamily property in `tailwind.config.js` to extend fonts
+```js
+{
+  fontFamily: {
+    'title-resource-rounded': ['ResourceHanRoundedCN-Bold', 'sans-serif'],
+    'body-harmony': ['HarmonyOSSans-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-resource-rounded text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-harmony text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Use subtle scale feedback on tap, such as `active:scale-95`, making elements feel gently pressed like soft candy.
+- For state changes, use `transition-all duration-200`. Delicate bounce, sway, or fade-in effects may be added, but avoid exaggerated motion and strong displacement.
+# Layout
+- Keep generous whitespace, clearly separate content sections, and use large rounded cards to hold information.
+- The main structure suits mobile: a simple top navigation or title area, a vertical card flow in the middle, and key action buttons fixed near the visual focus.
+- Card padding should feel spacious, commonly using `p-6`; use `rounded-2xl` and `rounded-3xl` for corners, and `rounded-full` for buttons.
+# Elements
+- Buttons use a soft pink background, white text, and a rounded pill shape: `bg-pink-400 text-white rounded-full shadow-md`.
+- Cards use white or light pink backgrounds with `border-2 border-pink-200` and soft shadows. On hover or touch, only enhance the shadow; do not use hard offset shadows.
+- Progress, completion states, habit tracking, and similar components can use dot groups, circular progress rings, or soft bars, keeping colors consistently pastel.
+- Decorative elements use semi-transparent dots, circles, and rounded floating blocks. Avoid sharp right angles, black backgrounds, neon glow effects, and heavy fonts.</t>
+        </is>
+      </c>
+      <c r="Z137" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>Airy Kawaii</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>Japanese kawaii meets minimalist whitespace: pastel, rounded, light, and gentle. The overall feel is like a soft breath of oxygen—friendly but not childish, cute but not cluttered.</t>
+        </is>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W138" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y138" t="inlineStr">
+        <is>
+          <t># Theme Name: Airy Kawaii
+# Vibe &amp; Description:
+Japanese kawaii meets minimalist whitespace: pastel, rounded, light, and gentle. The overall feel is like a soft breath of oxygen—friendly but not childish, cute but not cluttered.
+# Color
+- Use low-saturation pastel palettes; avoid dark backgrounds, fluorescent colors, and strong contrasts.
+- Backgrounds are mainly warm white and light cream (#FFF7ED / #FFF9F2). Use soft pink (#F9A8D4) as the primary color, with light purple (#A78BFA), light cyan (#67E8F9), and light yellow (#FDE68A) as accents. Text uses soft dark gray (#4B5563) to reduce the pressure of pure black.
+- Cards mostly use white or light pink backgrounds, with pale pastel borders such as #FBCFE8, creating a light, soft, and clean visual atmosphere.
+# Font
+- Use "ResourceHanRoundedCN-Bold" as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/ResourceHanRoundedCN-Bold.ttf)
+- Use "HarmonyOS Sans" as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/HarmonyOSSans_Regular.ttf)
+# Animation
+- Use subtle scale feedback on tap, such as `active:scale-95`, making elements feel gently pressed like soft candy.
+- For state changes, use `transition-all duration-200`. Delicate bounce, sway, or fade-in effects may be added, but avoid exaggerated motion and strong displacement.
+# Layout
+- Keep generous whitespace, clearly separate content sections, and use large rounded cards to hold information.
+- The main structure suits mobile: a simple top navigation or title area, a vertical card flow in the middle, and key action buttons fixed near the visual focus.
+- Card padding should feel spacious, commonly using `p-6`; use `rounded-2xl` and `rounded-3xl` for corners, and `rounded-full` for buttons.
+# Elements
+- Buttons use a soft pink background, white text, and a rounded pill shape: `bg-pink-400 text-white rounded-full shadow-md`.
+- Cards use white or light pink backgrounds with `border-2 border-pink-200` and soft shadows. On hover or touch, only enhance the shadow; do not use hard offset shadows.
+- Progress, completion states, habit tracking, and similar components can use dot groups, circular progress rings, or soft bars, keeping colors consistently pastel.
+- Decorative elements use semi-transparent dots, circles, and rounded floating blocks. Avoid sharp right angles, black backgrounds, neon glow effects, and heavy fonts.</t>
+        </is>
+      </c>
+      <c r="Z138" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>Minimal Executive</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>Classical serif typography, a cool-gray paper-textured background, and restrained blue accents create a quiet, refined, trustworthy business presence through fine lines, generous whitespace, and editorial-style composition.</t>
+        </is>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W139" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y139" t="inlineStr">
+        <is>
+          <t># Theme Name: Minimal Executive
+# Vibe &amp; Description:
+Classical serif typography, a cool-gray paper-textured background, and restrained blue accents create a quiet, refined, trustworthy business presence through fine lines, generous whitespace, and editorial-style composition.
+# Color
+- Keep the palette extremely restrained, using cool gray, deep black, pure white, and blue as the only accent color.
+- Use a cool-gray paper tone (#F9F9F9) for the background, deep black (#1A1A1A) for primary text, pure white (#FFFFFF) for card surfaces, and clear blue (#1C82F5) as the accent color. Avoid high saturation and harsh contrast overall, presenting the readability and elegance of a publication.
+# Font
+- Use "SourceHanSerifCN-SemiBold" as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-SemiBold.woff2)
+- Use "AlibabaPuHuiTi" as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'SourceHanSerifCN-SemiBold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-SemiBold.woff2' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the fontFamily property in `tailwind.config.js` to extend the fonts
+```js
+{
+  fontFamily: {
+    'title-serif-semibold': ['SourceHanSerifCN-SemiBold', 'serif'],
+    'body-alibaba': ['AlibabaPuHuiTi-Regular', 'sans-serif', 'serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-serif-semibold text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Motion is restrained, smooth, and bounce-free. Buttons rise or settle slightly on touch, while cards express state only through changes in shadow, border, and background brightness.
+- Elements appear with a slow fade-in of about 200-600ms, emphasizing a quiet, stable, editorial-grade reading rhythm.
+# Layout
+- Pages use generous whitespace and narrow content columns to create the reading feel of a premium publication. On mobile, maintain ample margins to avoid crowding information.
+- Use 1px cool-gray fine lines between sections to establish order. Titles are centered or arranged with subtle asymmetry, card spacing is relaxed, and body text line height remains airy.
+# Elements
+- Buttons use 6px corner radius. Primary buttons have a blue background with white text, while secondary buttons use a fine outlined style, with only slight brightness and shadow changes on interaction.
+- Cards use a white background, 8px corner radius, a fine gray border, and an extremely subtle shadow, with an optional 2px blue accent line at the top.
+- Section labels use small monospaced uppercase text with wide letter spacing, paired with fine lines extending across both sides to form a distinctive editorial structure.
+- The background may layer in extremely subtle paper noise and low-opacity blue glows, but it must remain clean, calm, and restrained.</t>
+        </is>
+      </c>
+      <c r="Z139" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>Minimal Executive</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>Classical serif typography, a cool-gray paper-textured background, and restrained blue accents create a quiet, refined, trustworthy business presence through fine lines, generous whitespace, and editorial-style composition.</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W140" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y140" t="inlineStr">
+        <is>
+          <t># Theme Name: Minimal Executive
+# Vibe &amp; Description:
+Classical serif typography, a cool-gray paper-textured background, and restrained blue accents create a quiet, refined, trustworthy business presence through fine lines, generous whitespace, and editorial-style composition.
+# Color
+- Keep the palette extremely restrained, using cool gray, deep black, pure white, and blue as the only accent color.
+- Use a cool-gray paper tone (#F9F9F9) for the background, deep black (#1A1A1A) for primary text, pure white (#FFFFFF) for card surfaces, and clear blue (#1C82F5) as the accent color. Avoid high saturation and harsh contrast overall, presenting the readability and elegance of a publication.
+# Font
+- Use "SourceHanSerifCN-SemiBold" as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-SemiBold.woff2)
+- Use "AlibabaPuHuiTi" as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- Motion is restrained, smooth, and bounce-free. Buttons rise or settle slightly on touch, while cards express state only through changes in shadow, border, and background brightness.
+- Elements appear with a slow fade-in of about 200-600ms, emphasizing a quiet, stable, editorial-grade reading rhythm.
+# Layout
+- Pages use generous whitespace and narrow content columns to create the reading feel of a premium publication. On mobile, maintain ample margins to avoid crowding information.
+- Use 1px cool-gray fine lines between sections to establish order. Titles are centered or arranged with subtle asymmetry, card spacing is relaxed, and body text line height remains airy.
+# Elements
+- Buttons use 6px corner radius. Primary buttons have a blue background with white text, while secondary buttons use a fine outlined style, with only slight brightness and shadow changes on interaction.
+- Cards use a white background, 8px corner radius, a fine gray border, and an extremely subtle shadow, with an optional 2px blue accent line at the top.
+- Section labels use small monospaced uppercase text with wide letter spacing, paired with fine lines extending across both sides to form a distinctive editorial structure.
+- The background may layer in extremely subtle paper noise and low-opacity blue glows, but it must remain clean, calm, and restrained.</t>
+        </is>
+      </c>
+      <c r="Z140" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>Comic Book Style</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>Thick black outlines, high-saturation print colors, irregular panels, and exaggerated motion create a sense of heat, adventure, and heroic storytelling.</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W141" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y141" t="inlineStr">
+        <is>
+          <t># Theme Name: Comic Book Style
+# Vibe &amp; Description:
+Thick black outlines, high-saturation print colors, irregular panels, and exaggerated motion create a sense of heat, adventure, and heroic storytelling.
+# Color
+- Use classic CMYK comic print colors for bright, high-contrast visuals.
+- Use paper white (#FFFEF0) or dark gray (#2C2C2C) for the background, and pure black (#000000) for text and outlines. Use comic red (#E23636), hero blue (#1E90FF), and warning yellow (#FFD700) as the main colors to emphasize impact, speed, and dramatic tension.
+# Font
+- Use "PangMenTitle" as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/PangMenTitle_Regular.ttf)
+- Use "AlibabaPuHuiTi" as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'PangMenTitle-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/PangMenTitle_Regular.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add a fontFamily property extension in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'title-pangmen': ['PangMenTitle-Regular', 'sans-serif'],
+    'body-alibaba': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-pangmen text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch, elements slightly scale or tilt, mimicking the pushed-in framing of comic panels. On tap, a brief burst star or “POW!” sound-effect text can appear.
+- When elements enter the page, use fast fly-in, bounce, or radiating-line spread animations to create the feeling of an action scene unfolding suddenly.
+# Layout
+- Use an irregular panel layout, with cards slightly tilted, overlapped, or breaking out of their frames to create a strong narrative rhythm.
+- Show important content in large panels or across sections, keep supporting content compact, and use diagonal composition and exaggerated perspective to enhance motion.
+# Elements
+- Cards and buttons use 2-4px thick black solid outlines, with corners that can feel slightly like hard comic cuts.
+- Speed lines: add radial speed lines around buttons, covers, or key information to strengthen the sense of motion.
+- Speech bubbles: prompts, tags, and notes can use oval or cloud-shaped bubbles with small tails preserved.
+- Halftone dots: layer circular dot textures over shadows, backgrounds, and transition areas to simulate a retro print feel.</t>
+        </is>
+      </c>
+      <c r="Z141" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>Comic Book Style</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>Thick black outlines, high-saturation print colors, irregular panels, and exaggerated motion create a sense of heat, adventure, and heroic storytelling.</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W142" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y142" t="inlineStr">
+        <is>
+          <t># Theme Name: Comic Book Style
+# Vibe &amp; Description:
+Thick black outlines, high-saturation print colors, irregular panels, and exaggerated motion create a sense of heat, adventure, and heroic storytelling.
+# Color
+- Use classic CMYK comic print colors for bright, high-contrast visuals.
+- Use paper white (#FFFEF0) or dark gray (#2C2C2C) for the background, and pure black (#000000) for text and outlines. Use comic red (#E23636), hero blue (#1E90FF), and warning yellow (#FFD700) as the main colors to emphasize impact, speed, and dramatic tension.
+# Font
+- Use "PangMenTitle" as the heading font. (https://resource-static.bj.bcebos.com/fonts-skill/PangMenTitle_Regular.ttf)
+- Use "AlibabaPuHuiTi" as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- On touch, elements slightly scale or tilt, mimicking the pushed-in framing of comic panels. On tap, a brief burst star or “POW!” sound-effect text can appear.
+- When elements enter the page, use fast fly-in, bounce, or radiating-line spread animations to create the feeling of an action scene unfolding suddenly.
+# Layout
+- Use an irregular panel layout, with cards slightly tilted, overlapped, or breaking out of their frames to create a strong narrative rhythm.
+- Show important content in large panels or across sections, keep supporting content compact, and use diagonal composition and exaggerated perspective to enhance motion.
+# Elements
+- Cards and buttons use 2-4px thick black solid outlines, with corners that can feel slightly like hard comic cuts.
+- Speed lines: add radial speed lines around buttons, covers, or key information to strengthen the sense of motion.
+- Speech bubbles: prompts, tags, and notes can use oval or cloud-shaped bubbles with small tails preserved.
+- Halftone dots: layer circular dot textures over shadows, backgrounds, and transition areas to simulate a retro print feel.</t>
+        </is>
+      </c>
+      <c r="Z142" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>Retro 90s</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>Early web and Windows 95 vibes, system fonts, highly saturated colorful elements, 3D beveled buttons, marquee text and under-construction energy, creating a rough, lively, anti-minimal nostalgic web feel.</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W143" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y143" t="inlineStr">
+        <is>
+          <t># Theme Name: Retro 90s
+# Vibe &amp; Description:
+Early web and Windows 95 vibes, system fonts, highly saturated colorful elements, 3D beveled buttons, marquee text and under-construction energy, creating a rough, lively, anti-minimal nostalgic web feel.
+# Color
+- Use high-contrast, highly saturated early system colors; avoid soft tones, translucency, and modern gradients.
+- Use Win95 gray (#C0C0C0) for the background, pure black (#000000) for text, pure blue (#0000FF) for links, purple (#800080) for visited, and red (#FF0000) for hover. Accent colors can use bright yellow (#FFFF00), bright green (#00FF00), and bright red (#FF0000); the title bar uses navy blue to bright blue (#000080 → #1084D0).
+# Font
+- Headings, “ZCOOLKuHei” (https://resource-static.bj.bcebos.com/fonts-skill/ZCOOLKuHei_Regular.ttf)
+- Body, “SourceHanSerifCN” (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'ZCOOLKuHei-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/ZCOOLKuHei_Regular.ttf' },
+  'SourceHanSerifCN-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2' },
+});
+```
+`tailwind.config.js` add the `fontFamily` property to extend the font set
+```js
+{
+  fontFamily: {
+    'zkkh-title': ['ZCOOLKuHei-Regular', 'sans-serif'],
+    'serif-body': ['SourceHanSerifCN-Regular', 'serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-zkkh-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-serif-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Motion is fast, direct, and digital, with no natural easing. When buttons are pressed, the bevel flips and shifts slightly, like a real system control being pushed.
+- Marquee text, rainbow loops, blinking “New!” badges, and jumping hit-counter digits can be used; stop looping animations under reduced motion.
+# Layout
+- Mobile uses a single-column stack, but keeps table-like borders, dense information, and horizontal scroll areas.
+- The page simulates a 90s web window: gray textured background, blue title bar, inset content area, visible grid lines, and grooved dividers. The layout does not chase minimal whitespace, but feels full, lively, and like an old web page carefully collaged together.
+# Elements
+- All buttons, cards, and input fields must use 0 corner radius and 2px beveled borders to distinguish raised and inset states.
+- Cards use a window style: blue gradient title bar, white bold title, gray outer frame, and a pale yellow or white content area.
+- Key areas use yellow-black caution stripes, paired with blinking badges, dynamic CTAs, or colorful block decorations.
+- Links are always underlined, keeping blue, purple, and red states without modern softening.
+- The background can layer a 45-degree tile texture, and dividers use a 3D etched effect with gray on top and white below.</t>
+        </is>
+      </c>
+      <c r="Z143" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>Retro 90s</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>Early web and Windows 95 vibes, system fonts, highly saturated colorful elements, 3D beveled buttons, marquee text and under-construction energy, creating a rough, lively, anti-minimal nostalgic web feel.</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W144" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y144" t="inlineStr">
+        <is>
+          <t># Theme Name: Retro 90s
+# Vibe &amp; Description:
+Early web and Windows 95 vibes, system fonts, highly saturated colorful elements, 3D beveled buttons, marquee text and under-construction energy, creating a rough, lively, anti-minimal nostalgic web feel.
+# Color
+- Use high-contrast, highly saturated early system colors; avoid soft tones, translucency, and modern gradients.
+- Use Win95 gray (#C0C0C0) for the background, pure black (#000000) for text, pure blue (#0000FF) for links, purple (#800080) for visited, and red (#FF0000) for hover. Accent colors can use bright yellow (#FFFF00), bright green (#00FF00), and bright red (#FF0000); the title bar uses navy blue to bright blue (#000080 → #1084D0).
+# Font
+- Headings, “ZCOOLKuHei” (https://resource-static.bj.bcebos.com/fonts-skill/ZCOOLKuHei_Regular.ttf)
+- Body, “SourceHanSerifCN” (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+# Animation
+- Motion is fast, direct, and digital, with no natural easing. When buttons are pressed, the bevel flips and shifts slightly, like a real system control being pushed.
+- Marquee text, rainbow loops, blinking “New!” badges, and jumping hit-counter digits can be used; stop looping animations under reduced motion.
+# Layout
+- Mobile uses a single-column stack, but keeps table-like borders, dense information, and horizontal scroll areas.
+- The page simulates a 90s web window: gray textured background, blue title bar, inset content area, visible grid lines, and grooved dividers. The layout does not chase minimal whitespace, but feels full, lively, and like an old web page carefully collaged together.
+# Elements
+- All buttons, cards, and input fields must use 0 corner radius and 2px beveled borders to distinguish raised and inset states.
+- Cards use a window style: blue gradient title bar, white bold title, gray outer frame, and a pale yellow or white content area.
+- Key areas use yellow-black caution stripes, paired with blinking badges, dynamic CTAs, or colorful block decorations.
+- Links are always underlined, keeping blue, purple, and red states without modern softening.
+- The background can layer a 45-degree tile texture, and dividers use a 3D etched effect with gray on top and white below.</t>
+        </is>
+      </c>
+      <c r="Z144" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>Quiet Couture</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>Quiet luxury in negative space, couture tailoring, low-saturation imagery, and hairline silver strokes create a restrained, immersive premium apparel browsing experience rich with fabric texture.</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W145" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y145" t="inlineStr">
+        <is>
+          <t># Theme Name: Quiet Couture
+# Vibe &amp; Description:
+Quiet luxury in negative space, couture tailoring, low-saturation imagery, and hairline silver strokes create a restrained, immersive premium apparel browsing experience rich with fabric texture.
+# Color
+- Strictly limit the palette, using only midnight black, pearl white, matte silver, oatmeal, and charcoal gray.
+- Use pearl white (#FDFBF7) or oatmeal (#F0EDE6) for backgrounds, midnight black (#111111) and charcoal gray (#2E2E2E) for text, and matte silver (#B0B2B8) for decorative lines. Avoid highly saturated colors, gradients, and heavy shadows, allowing garment materials and negative space to become the visual focus.
+# Font
+- Use "SourceHanSerifCN-Bold" as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use "AlibabaPuHuiTi" as the font for body text, navigation, and supporting text. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'SourceHanSerifCN-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the `fontFamily` property in `tailwind.config.js` to extend fonts
+```js
+{
+  fontFamily: {
+    'title-serif-bold': ['SourceHanSerifCN-Bold', 'serif'],
+    'body-alibaba': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-serif-bold text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- When elements appear, use a restrained “fade in + move up 24px” animation, lasting about 0.5s, to create a chapter-like feeling reminiscent of turning magazine pages.
+- When touching product images, apply only a slight scale-up, a hairline silver stroke reveal, or the appearance of “Explore / Preview” text, giving clear feedback without overpowering the content.
+# Layout
+- Use generous negative space to shape a sense of luxury, prioritizing spacing values in multiples of 8 such as 32px, 64px, and 96px.
+- Product content follows a chapter-based browsing flow, with each core section close to one screen in height and a single garment centered to emphasize silhouette and fabric texture.
+- Keep titles and decorative lines aligned, forming a quiet, precise visual order with an architectural feel.
+# Elements
+- Images use a low-saturation, high-contrast style, with pure white or light gray backgrounds to highlight material details such as wool, silk, and leather.
+- Buttons use transparent outline styling with midnight black borders; on touch, feedback appears through an expanding underline or a shift to matte silver.
+- Dividers, decorative lines, and hover boundaries consistently use 1px matte silver, avoiding thick borders, complex patterns, and heavy shadows.
+- Product cards avoid default shadows, relying on negative space, silver lines, and subtle scaling to establish hierarchy.</t>
+        </is>
+      </c>
+      <c r="Z145" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>Quiet Couture</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>Quiet luxury in negative space, couture tailoring, low-saturation imagery, and hairline silver strokes create a restrained, immersive premium apparel browsing experience rich with fabric texture.</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W146" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y146" t="inlineStr">
+        <is>
+          <t># Theme Name: Quiet Couture
+# Vibe &amp; Description:
+Quiet luxury in negative space, couture tailoring, low-saturation imagery, and hairline silver strokes create a restrained, immersive premium apparel browsing experience rich with fabric texture.
+# Color
+- Strictly limit the palette, using only midnight black, pearl white, matte silver, oatmeal, and charcoal gray.
+- Use pearl white (#FDFBF7) or oatmeal (#F0EDE6) for backgrounds, midnight black (#111111) and charcoal gray (#2E2E2E) for text, and matte silver (#B0B2B8) for decorative lines. Avoid highly saturated colors, gradients, and heavy shadows, allowing garment materials and negative space to become the visual focus.
+# Font
+- Use "SourceHanSerifCN-Bold" as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use "AlibabaPuHuiTi" as the font for body text, navigation, and supporting text. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- When elements appear, use a restrained “fade in + move up 24px” animation, lasting about 0.5s, to create a chapter-like feeling reminiscent of turning magazine pages.
+- When touching product images, apply only a slight scale-up, a hairline silver stroke reveal, or the appearance of “Explore / Preview” text, giving clear feedback without overpowering the content.
+# Layout
+- Use generous negative space to shape a sense of luxury, prioritizing spacing values in multiples of 8 such as 32px, 64px, and 96px.
+- Product content follows a chapter-based browsing flow, with each core section close to one screen in height and a single garment centered to emphasize silhouette and fabric texture.
+- Keep titles and decorative lines aligned, forming a quiet, precise visual order with an architectural feel.
+# Elements
+- Images use a low-saturation, high-contrast style, with pure white or light gray backgrounds to highlight material details such as wool, silk, and leather.
+- Buttons use transparent outline styling with midnight black borders; on touch, feedback appears through an expanding underline or a shift to matte silver.
+- Dividers, decorative lines, and hover boundaries consistently use 1px matte silver, avoiding thick borders, complex patterns, and heavy shadows.
+- Product cards avoid default shadows, relying on negative space, silver lines, and subtle scaling to establish hierarchy.</t>
+        </is>
+      </c>
+      <c r="Z146" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>Woven Texture</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>Linen, canvas, and denim-like textile textures, gentle neutrals, seam details, and soft shadows create a warm, touchable interface with a handmade feel.</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W147" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y147" t="inlineStr">
+        <is>
+          <t># Theme Name: Woven Texture
+# Vibe &amp; Description:
+Linen, canvas, and denim-like textile textures, gentle neutrals, seam details, and soft shadows create a warm, touchable interface with a handmade feel.
+# Color
+- Use linen, off-white, and warm gray as the main background tones; avoid pure white, pure black, and cool gray.
+- Use light textile tones (#F5F0E8, #FAF7F2, #EDE8E0) for the background, deep brown (#3D2E1E) or charcoal (#2C2C2C) for text, and warm gray (#8A7E72) for secondary text.
+- Keep accent colors to a minimum: terracotta red (#C47D5A), indigo (#4A6A7F), or mustard yellow (#D4A84B). Use warm brown (#C4B5A5) for borders and stitching, with low-opacity warm gray shadows.
+# Font
+- Use "Muyao Softbrush" as the title font to create a warm, handcrafted, human feel. (https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf)
+- Use "Source Han Serif CN" as the body font to ensure clear readability on the textile-texture background. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+## Font Import Method
+Load fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'MuyaoSoftbrush-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf' },
+  'SourceHanSerifCN-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2' },
+});
+```
+Add the `fontFamily` property to extend fonts in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'title-muyao': ['MuyaoSoftbrush-Regular', 'sans-serif'],
+    'body-serif': ['SourceHanSerifCN-Regular', 'serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-muyao text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-serif text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch, elements lift slightly, shadows deepen, and low-opacity highlights appear, as if light passes across the fabric. On click, they sink slightly, simulating soft fabric being pressed.
+- Keep motion gentle and restrained, around 180-260ms, avoiding large scale or bounce effects.
+# Layout
+- Use generous whitespace and soft sections; on mobile, favor a single-column layout and keep touch targets at no less than 44px.
+- Keep the background subtly textured at all times. Use texture density, shadow depth, and whitespace to build hierarchy, avoiding flat, textureless solid surfaces.
+# Elements
+- Buttons and cards use linen or off-white backgrounds, layered with subtle textile noise, and warm-brown solid or dashed stitching borders.
+- CTA elements can be designed in a fabric-label style, with 6-8px soft rounded corners, double stitching, or short thread-end accents.
+- Input fields use a light textile background and clear stitched borders; on focus, the border deepens slightly and gains a soft shadow.
+- Global texture can use `repeating-linear-gradient` to simulate warp and weft, then layer very low-opacity noise to create the feel of linen, canvas, or denim.</t>
+        </is>
+      </c>
+      <c r="Z147" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Woven Texture</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Linen, canvas, and denim-like textile textures, gentle neutrals, seam details, and soft shadows create a warm, touchable interface with a handmade feel.</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W148" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y148" t="inlineStr">
+        <is>
+          <t># Theme Name: Woven Texture
+# Vibe &amp; Description:
+Linen, canvas, and denim-like textile textures, gentle neutrals, seam details, and soft shadows create a warm, touchable interface with a handmade feel.
+# Color
+- Use linen, off-white, and warm gray as the main background tones; avoid pure white, pure black, and cool gray.
+- Use light textile tones (#F5F0E8, #FAF7F2, #EDE8E0) for the background, deep brown (#3D2E1E) or charcoal (#2C2C2C) for text, and warm gray (#8A7E72) for secondary text.
+- Keep accent colors to a minimum: terracotta red (#C47D5A), indigo (#4A6A7F), or mustard yellow (#D4A84B). Use warm brown (#C4B5A5) for borders and stitching, with low-opacity warm gray shadows.
+# Font
+- Use "Muyao Softbrush" as the title font to create a warm, handcrafted, human feel. (https://resource-static.bj.bcebos.com/fonts-skill/MuyaoSoftbrush_Regular.ttf)
+- Use "Source Han Serif CN" as the body font to ensure clear readability on the textile-texture background. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Regular.woff2)
+# Animation
+- On touch, elements lift slightly, shadows deepen, and low-opacity highlights appear, as if light passes across the fabric. On click, they sink slightly, simulating soft fabric being pressed.
+- Keep motion gentle and restrained, around 180-260ms, avoiding large scale or bounce effects.
+# Layout
+- Use generous whitespace and soft sections; on mobile, favor a single-column layout and keep touch targets at no less than 44px.
+- Keep the background subtly textured at all times. Use texture density, shadow depth, and whitespace to build hierarchy, avoiding flat, textureless solid surfaces.
+# Elements
+- Buttons and cards use linen or off-white backgrounds, layered with subtle textile noise, and warm-brown solid or dashed stitching borders.
+- CTA elements can be designed in a fabric-label style, with 6-8px soft rounded corners, double stitching, or short thread-end accents.
+- Input fields use a light textile background and clear stitched borders; on focus, the border deepens slightly and gains a soft shadow.
+- Global texture can use `repeating-linear-gradient` to simulate warp and weft, then layer very low-opacity noise to create the feel of linen, canvas, or denim.</t>
+        </is>
+      </c>
+      <c r="Z148" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>Candy Brutalism</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>Hard-edged structure, saturated candy colors, thick black outlines, and pronounced offset shadows. The overall look is bold and playful yet clearly ordered, like an interface built from colorful blocks.</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W149" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y149" t="inlineStr">
+        <is>
+          <t># Theme Name: Candy Brutalism
+# Vibe &amp; Description:
+Hard-edged structure, saturated candy colors, thick black outlines, and pronounced offset shadows. The overall look is bold and playful yet clearly ordered, like an interface built from colorful blocks.
+# Color
+- Use highly saturated solid colors as the main visual language, avoiding soft pastels, low-saturation tones, and large gradients.
+- Keep the background mainly white or light (#FFFFFF), with core color blocks in pink (#FF6B9D), yellow (#FFD93D), blue (#6BCBFF), and green (#6BCB77). Use black or dark gray (#1A1A1A / #2D2D2D) for text, borders, and shadows to create a strong, direct, and clear visual contrast.
+# Font
+- Use "YouSheBiaoTiHei" as the heading font, emphasizing weight, sturdiness, and a poster-like feel. (https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf)
+- Use "Alibaba PuHuiTi 3.0" as the body font, maintaining a bold, crisp, direct reading experience. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'YouSheBiaoTiHei-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Extend fonts by adding the fontFamily property in `tailwind.config.js`
+```js
+{
+  fontFamily: {
+    'youshe-title': ['YouSheBiaoTiHei-Regular', 'sans-serif'],
+    'alibaba-puhuiti-body': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-youshe-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-alibaba-puhuiti-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- When touched, elements lift slightly or rotate (-2deg to 2deg), with stronger shadow offset, creating direct, forceful feedback.
+- On tap, elements sink 2-4px, shadows snap tighter, and transitions stay within 120-200ms to avoid soft, sluggish, or overly elastic motion.
+# Layout
+- The page uses a clear hard-edge grid and color-block sections, with information areas joined together as neatly as building blocks.
+- Cards, buttons, and key modules use 2-4px black solid borders, paired with solid offset shadows of 4px or more, maintaining strong hierarchy and a sense of order.
+# Elements
+- Buttons and cards use saturated color blocks, thick black borders, and blur-free offset shadows to form signature neo-brutalist components.
+- Sticker, hand-drawn arrow, star, and circle doodles can be added to increase playfulness, but they must not compromise layout clarity.
+- The background may include a small amount of noise or striped texture to enhance tactility, but frosted glass, blurred shadows, and complex gradients are prohibited.
+- All interactive elements should remain solid, hard-edged, and strongly clickable, with mobile touch targets no smaller than 44px.</t>
+        </is>
+      </c>
+      <c r="Z149" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Candy Brutalism</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Hard-edged structure, saturated candy colors, thick black outlines, and pronounced offset shadows. The overall look is bold and playful yet clearly ordered, like an interface built from colorful blocks.</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W150" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y150" t="inlineStr">
+        <is>
+          <t># Theme Name: Candy Brutalism
+# Vibe &amp; Description:
+Hard-edged structure, saturated candy colors, thick black outlines, and pronounced offset shadows. The overall look is bold and playful yet clearly ordered, like an interface built from colorful blocks.
+# Color
+- Use highly saturated solid colors as the main visual language, avoiding soft pastels, low-saturation tones, and large gradients.
+- Keep the background mainly white or light (#FFFFFF), with core color blocks in pink (#FF6B9D), yellow (#FFD93D), blue (#6BCBFF), and green (#6BCB77). Use black or dark gray (#1A1A1A / #2D2D2D) for text, borders, and shadows to create a strong, direct, and clear visual contrast.
+# Font
+- Use "YouSheBiaoTiHei" as the heading font, emphasizing weight, sturdiness, and a poster-like feel. (https://resource-static.bj.bcebos.com/fonts-skill/YouSheBiaoTiHei_Regular.ttf)
+- Use "Alibaba PuHuiTi 3.0" as the body font, maintaining a bold, crisp, direct reading experience. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- When touched, elements lift slightly or rotate (-2deg to 2deg), with stronger shadow offset, creating direct, forceful feedback.
+- On tap, elements sink 2-4px, shadows snap tighter, and transitions stay within 120-200ms to avoid soft, sluggish, or overly elastic motion.
+# Layout
+- The page uses a clear hard-edge grid and color-block sections, with information areas joined together as neatly as building blocks.
+- Cards, buttons, and key modules use 2-4px black solid borders, paired with solid offset shadows of 4px or more, maintaining strong hierarchy and a sense of order.
+# Elements
+- Buttons and cards use saturated color blocks, thick black borders, and blur-free offset shadows to form signature neo-brutalist components.
+- Sticker, hand-drawn arrow, star, and circle doodles can be added to increase playfulness, but they must not compromise layout clarity.
+- The background may include a small amount of noise or striped texture to enhance tactility, but frosted glass, blurred shadows, and complex gradients are prohibited.
+- All interactive elements should remain solid, hard-edged, and strongly clickable, with mobile touch targets no smaller than 44px.</t>
+        </is>
+      </c>
+      <c r="Z150" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Art Nouveau</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Organic curves, vines and florals, and Mucha poster-inspired ornamentation, using a deep green, gold, and ivory palette to emphasize elegance, nature, and an artful sense of flowing beauty.</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W151" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y151" t="inlineStr">
+        <is>
+          <t># Theme Name: Art Nouveau
+# Vibe &amp; Description:
+Organic curves, vines and florals, and Mucha poster-inspired ornamentation, using a deep green, gold, and ivory palette to emphasize elegance, nature, and an artful sense of flowing beauty.
+# Color
+- Use deep green, gold, ivory, and warm brown; avoid pure black, neon colors, and highly saturated fluorescent colors.
+- Use ivory (#F5F0E1) or light ivory layers (#FAF7EF) for backgrounds, deep green (#2D5016) or dark brown for text, and gold (#C9A227) for accents and borders. The overall palette should feel like a vintage exhibition poster: soft, refined, and naturally ornamental.
+# Font
+- Use “SourceHanSerifCN-Bold” as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use “AlibabaPuHuiTi” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'SourceHanSerifCN-Bold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the fontFamily property to `tailwind.config.js` to extend the fonts
+```js
+{
+  fontFamily: {
+    'title-serif-bold': ['SourceHanSerifCN-Bold', 'serif'],
+    'body-alibaba': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-title-serif-bold text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-body-alibaba text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- On touch, elements lift slightly and reveal a soft golden glow, like light passing over a gold-foil border.
+- Elements appear with a slow fade-in and subtle displacement; floral and vine decorations may use low-speed floating or unfurling animations, keeping the overall rhythm soft and elegant.
+# Layout
+- Use an asymmetrical composition, with titles and decorative graphics forming a 60/40 visual relationship to create vintage poster-like layering.
+- Cards and sections should maintain generous whitespace, using rounded corners, thin gold borders, and soft shadows. On mobile, prioritize a single-column layout, with floral dividers added locally to enhance rhythm.
+# Elements
+- Buttons and cards use `rounded-2xl` or `rounded-full`, paired with `border-2 border-[#C9A227]/60` and soft shadows.
+- Vine patterns: use SVGs or background patterns as decorations for titles, dividers, and card corners.
+- Floral borders: key areas may include circular floral frames or Mucha-style arched ornamentation.
+- Emphasized text: use a light deep-green background texture or a gold underline, keeping it refined without drawing excessive attention.</t>
+        </is>
+      </c>
+      <c r="Z151" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Art Nouveau</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>Organic curves, vines and florals, and Mucha poster-inspired ornamentation, using a deep green, gold, and ivory palette to emphasize elegance, nature, and an artful sense of flowing beauty.</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W152" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y152" t="inlineStr">
+        <is>
+          <t># Theme Name: Art Nouveau
+# Vibe &amp; Description:
+Organic curves, vines and florals, and Mucha poster-inspired ornamentation, using a deep green, gold, and ivory palette to emphasize elegance, nature, and an artful sense of flowing beauty.
+# Color
+- Use deep green, gold, ivory, and warm brown; avoid pure black, neon colors, and highly saturated fluorescent colors.
+- Use ivory (#F5F0E1) or light ivory layers (#FAF7EF) for backgrounds, deep green (#2D5016) or dark brown for text, and gold (#C9A227) for accents and borders. The overall palette should feel like a vintage exhibition poster: soft, refined, and naturally ornamental.
+# Font
+- Use “SourceHanSerifCN-Bold” as the title font. (https://resource-static.bj.bcebos.com/fonts-skill/SourceHanSerifCN-Bold.woff2)
+- Use “AlibabaPuHuiTi” as the body font. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- On touch, elements lift slightly and reveal a soft golden glow, like light passing over a gold-foil border.
+- Elements appear with a slow fade-in and subtle displacement; floral and vine decorations may use low-speed floating or unfurling animations, keeping the overall rhythm soft and elegant.
+# Layout
+- Use an asymmetrical composition, with titles and decorative graphics forming a 60/40 visual relationship to create vintage poster-like layering.
+- Cards and sections should maintain generous whitespace, using rounded corners, thin gold borders, and soft shadows. On mobile, prioritize a single-column layout, with floral dividers added locally to enhance rhythm.
+# Elements
+- Buttons and cards use `rounded-2xl` or `rounded-full`, paired with `border-2 border-[#C9A227]/60` and soft shadows.
+- Vine patterns: use SVGs or background patterns as decorations for titles, dividers, and card corners.
+- Floral borders: key areas may include circular floral frames or Mucha-style arched ornamentation.
+- Emphasized text: use a light deep-green background texture or a gold underline, keeping it refined without drawing excessive attention.</t>
+        </is>
+      </c>
+      <c r="Z152" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Neon Tech</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>High-saturation neon on a dark base, with glassmorphism glows and layered color gradients, creating a modern, energetic, cutting-edge digital tech feel.</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="W153" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y153" t="inlineStr">
+        <is>
+          <t># Theme Name: Neon Tech
+# Vibe &amp; Description:
+High-saturation neon on a dark base, with glassmorphism glows and layered color gradients, creating a modern, energetic, cutting-edge digital tech feel.
+# Color
+- Use deep purple-blue as the overall background base; recommend `#1e1b4b` or a similar dark tone. Do not use pure white backgrounds, gray backgrounds, or black text.
+- Use purple `#8b5cf6` as the primary color, paired with cyan `#06b6d4`, rose `#ec4899`, and amber `#f59e0b` as accents.
+- Use gradients for large visual emphasis: `from-violet-500 via-purple-500 to-fuchsia-500`, for buttons, title accents, decorative lines, and key numbers.
+- Use a semi-transparent glass effect for cards: `bg-white/10`, `border-white/20`, with `text-white`, `text-white/80`, and `text-white/60` to preserve hierarchy.
+# Font
+- Use "Alibaba PuHuiTi" as the title font to emphasize the tech feel and information hierarchy. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_SemiBold.ttf)
+- Use "Alibaba PuHuiTi" as the body font to keep it clear, modern, and readable. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+## Font Import Method
+Load the fonts in `app/_layout.tsx`
+```js
+import { useFonts } from 'expo-font';
+const [fontsLoaded] = useFonts({
+  'AlibabaPuHuiTi-SemiBold': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_SemiBold.ttf' },
+  'AlibabaPuHuiTi-Regular': { uri: 'https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf' },
+});
+```
+Add the `fontFamily` property in `tailwind.config.js` to extend the fonts
+```js
+{
+  fontFamily: {
+    'alibaba-puhuiti-title': ['AlibabaPuHuiTi-SemiBold', 'sans-serif'],
+    'alibaba-puhuiti-body': ['AlibabaPuHuiTi-Regular', 'sans-serif'],
+  }
+}
+```
+## Code Example
+```jsx
+&lt;Text className="font-alibaba-puhuiti-title text-3xl"&gt;&lt;/Text&gt;
+&lt;Text className="font-alibaba-puhuiti-body text-base"&gt;&lt;/Text&gt;
+```
+# Animation
+- Use subtle scaling feedback when buttons or cards are tapped: `active:scale-95`, paired with enhanced colored shadows to create a clear touch response.
+- When elements appear, use a "fade in + glow spread" effect; gradient accents can float slowly to create a dynamic tech atmosphere.
+- Keep all interactions smooth: `transition-all duration-300`, avoiding abrupt shifts and traditional hard-edged shadows.
+# Layout
+- Build the page on a dark full-screen background, with a simple logo and primary action entry at the top, and vertically scrolling content below.
+- Make the hero area stand out with a large title, subtitle, and main CTA, with blurred gradient glow orbs layered in the background to create a focal point.
+- Present features, data, and reviews in vertically stacked glass cards, with generous spacing between cards and a clear mobile reading rhythm.
+# Elements
+- Use a purple-to-rose gradient background for buttons, with `rounded-2xl` corners and a colored glow shadow: `shadow-violet-500/30`.
+- Use `rounded-3xl`, semi-transparent backgrounds, thin white borders, and `backdrop-blur-xl` for cards to create a floating glass feel.
+- Use gradient text for key numbers, and add cyan, light purple, or rose accents to titles and icons.
+- Use blurred colored spots, gradient lines, and semi-transparent overlays for background decoration, avoiding solid white cards, black text, and sharp corners.</t>
+        </is>
+      </c>
+      <c r="Z153" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>任思远</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Neon Tech</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>High-saturation neon on a dark base, with glassmorphism glows and layered color gradients, creating a modern, energetic, cutting-edge digital tech feel.</t>
+        </is>
+      </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>Web, MiniProgram</t>
+        </is>
+      </c>
+      <c r="W154" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y154" t="inlineStr">
+        <is>
+          <t># Theme Name: Neon Tech
+# Vibe &amp; Description:
+High-saturation neon on a dark base, with glassmorphism glows and layered color gradients, creating a modern, energetic, cutting-edge digital tech feel.
+# Color
+- Use deep purple-blue as the overall background base; recommend `#1e1b4b` or a similar dark tone. Do not use pure white backgrounds, gray backgrounds, or black text.
+- Use purple `#8b5cf6` as the primary color, paired with cyan `#06b6d4`, rose `#ec4899`, and amber `#f59e0b` as accents.
+- Use gradients for large visual emphasis: `from-violet-500 via-purple-500 to-fuchsia-500`, for buttons, title accents, decorative lines, and key numbers.
+- Use a semi-transparent glass effect for cards: `bg-white/10`, `border-white/20`, with `text-white`, `text-white/80`, and `text-white/60` to preserve hierarchy.
+# Font
+- Use "Alibaba PuHuiTi" as the title font to emphasize the tech feel and information hierarchy. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_SemiBold.ttf)
+- Use "Alibaba PuHuiTi" as the body font to keep it clear, modern, and readable. (https://resource-static.bj.bcebos.com/fonts-skill/AlibabaPuHuiTi_Regular.ttf)
+# Animation
+- Use subtle scaling feedback when buttons or cards are tapped: `active:scale-95`, paired with enhanced colored shadows to create a clear touch response.
+- When elements appear, use a "fade in + glow spread" effect; gradient accents can float slowly to create a dynamic tech atmosphere.
+- Keep all interactions smooth: `transition-all duration-300`, avoiding abrupt shifts and traditional hard-edged shadows.
+# Layout
+- Build the page on a dark full-screen background, with a simple logo and primary action entry at the top, and vertically scrolling content below.
+- Make the hero area stand out with a large title, subtitle, and main CTA, with blurred gradient glow orbs layered in the background to create a focal point.
+- Present features, data, and reviews in vertically stacked glass cards, with generous spacing between cards and a clear mobile reading rhythm.
+# Elements
+- Use a purple-to-rose gradient background for buttons, with `rounded-2xl` corners and a colored glow shadow: `shadow-violet-500/30`.
+- Use `rounded-3xl`, semi-transparent backgrounds, thin white borders, and `backdrop-blur-xl` for cards to create a floating glass feel.
+- Use gradient text for key numbers, and add cyan, light purple, or rose accents to titles and icons.
+- Use blurred colored spots, gradient lines, and semi-transparent overlays for background decoration, avoiding solid white cards, black text, and sharp corners.</t>
+        </is>
+      </c>
+      <c r="Z154" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:59:38</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>